<commit_message>
Add generated leaderboard data - 2024-03-30T19:07:29
</commit_message>
<xml_diff>
--- a/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
+++ b/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
@@ -134,7 +134,7 @@
     <t>shahid24</t>
   </si>
   <si>
-    <t>58.5%</t>
+    <t>58.55%</t>
   </si>
   <si>
     <t>22R01A0531</t>
@@ -227,7 +227,7 @@
     <t>22r01a05l1</t>
   </si>
   <si>
-    <t>44.21%</t>
+    <t>44.22%</t>
   </si>
   <si>
     <t>22R01A05K7</t>
@@ -269,7 +269,7 @@
     <t>@msaiteja665</t>
   </si>
   <si>
-    <t>43.15%</t>
+    <t>43.18%</t>
   </si>
   <si>
     <t>22R01A73B1</t>
@@ -614,7 +614,7 @@
     <t>nooreen_44</t>
   </si>
   <si>
-    <t>33.31%</t>
+    <t>33.59%</t>
   </si>
   <si>
     <t>22R01A04G5</t>
@@ -1232,7 +1232,7 @@
     <t>pullurusaketh</t>
   </si>
   <si>
-    <t>24.37%</t>
+    <t>24.41%</t>
   </si>
   <si>
     <t>22R01A0484</t>
@@ -1307,7 +1307,7 @@
     <t>@KIREET_5L5</t>
   </si>
   <si>
-    <t>22.81%</t>
+    <t>22.82%</t>
   </si>
   <si>
     <t>22R01A67H4</t>
@@ -5582,88 +5582,91 @@
     <t>0.4%</t>
   </si>
   <si>
+    <t>22R01A0415</t>
+  </si>
+  <si>
+    <t>22r01a0415</t>
+  </si>
+  <si>
+    <t>Codechrfcmrithyderabad</t>
+  </si>
+  <si>
+    <t>22R01A67K2</t>
+  </si>
+  <si>
+    <t>22r01apnwy</t>
+  </si>
+  <si>
+    <t>22r01a67k2</t>
+  </si>
+  <si>
+    <t>c22r01a67k2</t>
+  </si>
+  <si>
+    <t>22R01A04A1</t>
+  </si>
+  <si>
+    <t>cmrit26_22_4a1</t>
+  </si>
+  <si>
+    <t>22r01a04a1</t>
+  </si>
+  <si>
+    <t>0.37%</t>
+  </si>
+  <si>
+    <t>22R01A04F4</t>
+  </si>
+  <si>
+    <t>22r01a04f4</t>
+  </si>
+  <si>
+    <t>sathwik_f4</t>
+  </si>
+  <si>
+    <t>22R01A04A9</t>
+  </si>
+  <si>
+    <t>22r01a04a9</t>
+  </si>
+  <si>
+    <t>0.34%</t>
+  </si>
+  <si>
+    <t>22R01A04D6</t>
+  </si>
+  <si>
+    <t>ARCHANA</t>
+  </si>
+  <si>
+    <t>23R05A0414</t>
+  </si>
+  <si>
+    <t>Vennela_L14</t>
+  </si>
+  <si>
+    <t>23r05a0414</t>
+  </si>
+  <si>
+    <t>vennela_414</t>
+  </si>
+  <si>
+    <t>22R01A0475</t>
+  </si>
+  <si>
+    <t>22r01a0475</t>
+  </si>
+  <si>
+    <t>cmr22r01a0475</t>
+  </si>
+  <si>
     <t>22R01A7318</t>
   </si>
   <si>
     <t>22r01a7318</t>
   </si>
   <si>
-    <t>22R01A0415</t>
-  </si>
-  <si>
-    <t>22r01a0415</t>
-  </si>
-  <si>
-    <t>Codechrfcmrithyderabad</t>
-  </si>
-  <si>
-    <t>22R01A67K2</t>
-  </si>
-  <si>
-    <t>22r01apnwy</t>
-  </si>
-  <si>
-    <t>22r01a67k2</t>
-  </si>
-  <si>
-    <t>c22r01a67k2</t>
-  </si>
-  <si>
-    <t>22R01A04A1</t>
-  </si>
-  <si>
-    <t>cmrit26_22_4a1</t>
-  </si>
-  <si>
-    <t>22r01a04a1</t>
-  </si>
-  <si>
-    <t>0.37%</t>
-  </si>
-  <si>
-    <t>22R01A04F4</t>
-  </si>
-  <si>
-    <t>22r01a04f4</t>
-  </si>
-  <si>
-    <t>sathwik_f4</t>
-  </si>
-  <si>
-    <t>22R01A04A9</t>
-  </si>
-  <si>
-    <t>22r01a04a9</t>
-  </si>
-  <si>
-    <t>0.34%</t>
-  </si>
-  <si>
-    <t>22R01A04D6</t>
-  </si>
-  <si>
-    <t>ARCHANA</t>
-  </si>
-  <si>
-    <t>23R05A0414</t>
-  </si>
-  <si>
-    <t>Vennela_L14</t>
-  </si>
-  <si>
-    <t>23r05a0414</t>
-  </si>
-  <si>
-    <t>vennela_414</t>
-  </si>
-  <si>
-    <t>22R01A0475</t>
-  </si>
-  <si>
-    <t>22r01a0475</t>
-  </si>
-  <si>
-    <t>cmr22r01a0475</t>
+    <t>0.29%</t>
   </si>
   <si>
     <t>22R01A6775</t>
@@ -5673,9 +5676,6 @@
   </si>
   <si>
     <t>Samanvitha10</t>
-  </si>
-  <si>
-    <t>0.29%</t>
   </si>
   <si>
     <t>23R05A6714</t>
@@ -9914,7 +9914,7 @@
         <v>94.0</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>60.0</v>
+        <v>65.0</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>38</v>
@@ -10178,7 +10178,7 @@
         <v>30.0</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>79.0</v>
+        <v>80.0</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>68</v>
@@ -10266,7 +10266,7 @@
         <v>108.0</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>101.0</v>
+        <v>104.0</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>82</v>
@@ -11296,7 +11296,7 @@
         <v>197</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>13.0</v>
+        <v>18.0</v>
       </c>
       <c r="N38" s="2" t="s">
         <v>200</v>
@@ -13214,7 +13214,7 @@
         <v>27.0</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="H82" s="2" t="s">
         <v>403</v>
@@ -13390,7 +13390,7 @@
         <v>30.0</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>61.0</v>
+        <v>62.0</v>
       </c>
       <c r="H86" s="2" t="s">
         <v>428</v>
@@ -26798,7 +26798,7 @@
         <v>1856</v>
       </c>
       <c r="C391" s="2" t="s">
-        <v>80</v>
+        <v>1857</v>
       </c>
       <c r="D391" s="2" t="n">
         <v>0.0</v>
@@ -26819,7 +26819,7 @@
         <v>0.0</v>
       </c>
       <c r="J391" s="2" t="s">
-        <v>1857</v>
+        <v>1858</v>
       </c>
       <c r="K391" s="2" t="n">
         <v>0.0</v>
@@ -26839,16 +26839,16 @@
         <v>391.0</v>
       </c>
       <c r="B392" s="2" t="s">
-        <v>1858</v>
+        <v>1859</v>
       </c>
       <c r="C392" s="2" t="s">
-        <v>1859</v>
+        <v>80</v>
       </c>
       <c r="D392" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E392" s="2" t="s">
-        <v>1859</v>
+        <v>1860</v>
       </c>
       <c r="F392" s="2" t="n">
         <v>0.0</v>
@@ -26857,19 +26857,19 @@
         <v>0.0</v>
       </c>
       <c r="H392" s="2" t="s">
-        <v>1859</v>
+        <v>1861</v>
       </c>
       <c r="I392" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J392" s="2" t="s">
-        <v>1860</v>
+        <v>1862</v>
       </c>
       <c r="K392" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="L392" s="2" t="s">
-        <v>1859</v>
+        <v>1861</v>
       </c>
       <c r="M392" s="2" t="n">
         <v>7.0</v>
@@ -26883,25 +26883,25 @@
         <v>392.0</v>
       </c>
       <c r="B393" s="2" t="s">
-        <v>1861</v>
+        <v>1863</v>
       </c>
       <c r="C393" s="2" t="s">
-        <v>80</v>
+        <v>1864</v>
       </c>
       <c r="D393" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E393" s="2" t="s">
-        <v>1862</v>
+        <v>1865</v>
       </c>
       <c r="F393" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G393" s="2" t="n">
-        <v>0.0</v>
+        <v>3.0</v>
       </c>
       <c r="H393" s="2" t="s">
-        <v>1863</v>
+        <v>1865</v>
       </c>
       <c r="I393" s="2" t="n">
         <v>0.0</v>
@@ -26913,13 +26913,13 @@
         <v>0.0</v>
       </c>
       <c r="L393" s="2" t="s">
-        <v>1863</v>
+        <v>1865</v>
       </c>
       <c r="M393" s="2" t="n">
-        <v>7.0</v>
+        <v>6.0</v>
       </c>
       <c r="N393" s="2" t="s">
-        <v>1855</v>
+        <v>1866</v>
       </c>
     </row>
     <row r="394">
@@ -26927,16 +26927,16 @@
         <v>393.0</v>
       </c>
       <c r="B394" s="2" t="s">
-        <v>1865</v>
+        <v>1867</v>
       </c>
       <c r="C394" s="2" t="s">
-        <v>1866</v>
+        <v>1868</v>
       </c>
       <c r="D394" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E394" s="2" t="s">
-        <v>1867</v>
+        <v>1868</v>
       </c>
       <c r="F394" s="2" t="n">
         <v>0.0</v>
@@ -26945,25 +26945,25 @@
         <v>3.0</v>
       </c>
       <c r="H394" s="2" t="s">
-        <v>1867</v>
+        <v>1869</v>
       </c>
       <c r="I394" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J394" s="2" t="s">
-        <v>1866</v>
+        <v>1869</v>
       </c>
       <c r="K394" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="L394" s="2" t="s">
-        <v>1867</v>
+        <v>1868</v>
       </c>
       <c r="M394" s="2" t="n">
         <v>6.0</v>
       </c>
       <c r="N394" s="2" t="s">
-        <v>1868</v>
+        <v>1866</v>
       </c>
     </row>
     <row r="395">
@@ -26971,43 +26971,43 @@
         <v>394.0</v>
       </c>
       <c r="B395" s="2" t="s">
-        <v>1869</v>
+        <v>1870</v>
       </c>
       <c r="C395" s="2" t="s">
-        <v>1870</v>
+        <v>80</v>
       </c>
       <c r="D395" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E395" s="2" t="s">
-        <v>1870</v>
+        <v>80</v>
       </c>
       <c r="F395" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G395" s="2" t="n">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="H395" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="I395" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J395" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="K395" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L395" s="2" t="s">
         <v>1871</v>
-      </c>
-      <c r="I395" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J395" s="2" t="s">
-        <v>1871</v>
-      </c>
-      <c r="K395" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="L395" s="2" t="s">
-        <v>1870</v>
       </c>
       <c r="M395" s="2" t="n">
         <v>6.0</v>
       </c>
       <c r="N395" s="2" t="s">
-        <v>1868</v>
+        <v>1872</v>
       </c>
     </row>
     <row r="396">
@@ -27015,7 +27015,7 @@
         <v>395.0</v>
       </c>
       <c r="B396" s="2" t="s">
-        <v>1872</v>
+        <v>1873</v>
       </c>
       <c r="C396" s="2" t="s">
         <v>80</v>
@@ -27024,7 +27024,7 @@
         <v>0.0</v>
       </c>
       <c r="E396" s="2" t="s">
-        <v>80</v>
+        <v>1873</v>
       </c>
       <c r="F396" s="2" t="n">
         <v>0.0</v>
@@ -27033,13 +27033,13 @@
         <v>0.0</v>
       </c>
       <c r="H396" s="2" t="s">
-        <v>80</v>
+        <v>1874</v>
       </c>
       <c r="I396" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J396" s="2" t="s">
-        <v>80</v>
+        <v>1873</v>
       </c>
       <c r="K396" s="2" t="n">
         <v>0.0</v>
@@ -27051,7 +27051,7 @@
         <v>6.0</v>
       </c>
       <c r="N396" s="2" t="s">
-        <v>1874</v>
+        <v>1872</v>
       </c>
     </row>
     <row r="397">
@@ -27062,13 +27062,13 @@
         <v>1875</v>
       </c>
       <c r="C397" s="2" t="s">
-        <v>80</v>
+        <v>1876</v>
       </c>
       <c r="D397" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E397" s="2" t="s">
-        <v>1875</v>
+        <v>80</v>
       </c>
       <c r="F397" s="2" t="n">
         <v>0.0</v>
@@ -27077,25 +27077,25 @@
         <v>0.0</v>
       </c>
       <c r="H397" s="2" t="s">
-        <v>1876</v>
+        <v>1877</v>
       </c>
       <c r="I397" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J397" s="2" t="s">
-        <v>1875</v>
+        <v>1878</v>
       </c>
       <c r="K397" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="L397" s="2" t="s">
-        <v>1875</v>
+        <v>1877</v>
       </c>
       <c r="M397" s="2" t="n">
         <v>6.0</v>
       </c>
       <c r="N397" s="2" t="s">
-        <v>1874</v>
+        <v>1872</v>
       </c>
     </row>
     <row r="398">
@@ -27103,16 +27103,16 @@
         <v>397.0</v>
       </c>
       <c r="B398" s="2" t="s">
-        <v>1877</v>
+        <v>1879</v>
       </c>
       <c r="C398" s="2" t="s">
-        <v>1878</v>
+        <v>80</v>
       </c>
       <c r="D398" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E398" s="2" t="s">
-        <v>80</v>
+        <v>1880</v>
       </c>
       <c r="F398" s="2" t="n">
         <v>0.0</v>
@@ -27121,25 +27121,25 @@
         <v>0.0</v>
       </c>
       <c r="H398" s="2" t="s">
-        <v>1879</v>
+        <v>1880</v>
       </c>
       <c r="I398" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J398" s="2" t="s">
+        <v>1881</v>
+      </c>
+      <c r="K398" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L398" s="2" t="s">
         <v>1880</v>
-      </c>
-      <c r="K398" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="L398" s="2" t="s">
-        <v>1879</v>
       </c>
       <c r="M398" s="2" t="n">
         <v>6.0</v>
       </c>
       <c r="N398" s="2" t="s">
-        <v>1874</v>
+        <v>1872</v>
       </c>
     </row>
     <row r="399">
@@ -27147,7 +27147,7 @@
         <v>398.0</v>
       </c>
       <c r="B399" s="2" t="s">
-        <v>1881</v>
+        <v>1882</v>
       </c>
       <c r="C399" s="2" t="s">
         <v>80</v>
@@ -27156,7 +27156,7 @@
         <v>0.0</v>
       </c>
       <c r="E399" s="2" t="s">
-        <v>1882</v>
+        <v>1883</v>
       </c>
       <c r="F399" s="2" t="n">
         <v>0.0</v>
@@ -27165,7 +27165,7 @@
         <v>0.0</v>
       </c>
       <c r="H399" s="2" t="s">
-        <v>1882</v>
+        <v>1883</v>
       </c>
       <c r="I399" s="2" t="n">
         <v>0.0</v>
@@ -27177,13 +27177,13 @@
         <v>0.0</v>
       </c>
       <c r="L399" s="2" t="s">
-        <v>1882</v>
+        <v>1883</v>
       </c>
       <c r="M399" s="2" t="n">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="N399" s="2" t="s">
-        <v>1874</v>
+        <v>1884</v>
       </c>
     </row>
     <row r="400">
@@ -27191,16 +27191,16 @@
         <v>399.0</v>
       </c>
       <c r="B400" s="2" t="s">
-        <v>1884</v>
+        <v>1885</v>
       </c>
       <c r="C400" s="2" t="s">
-        <v>1885</v>
+        <v>1886</v>
       </c>
       <c r="D400" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E400" s="2" t="s">
-        <v>1885</v>
+        <v>1886</v>
       </c>
       <c r="F400" s="2" t="n">
         <v>0.0</v>
@@ -27209,25 +27209,25 @@
         <v>0.0</v>
       </c>
       <c r="H400" s="2" t="s">
+        <v>1887</v>
+      </c>
+      <c r="I400" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J400" s="2" t="s">
         <v>1886</v>
       </c>
-      <c r="I400" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J400" s="2" t="s">
-        <v>1885</v>
-      </c>
       <c r="K400" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="L400" s="2" t="s">
-        <v>1885</v>
+        <v>1886</v>
       </c>
       <c r="M400" s="2" t="n">
         <v>5.0</v>
       </c>
       <c r="N400" s="2" t="s">
-        <v>1887</v>
+        <v>1884</v>
       </c>
     </row>
     <row r="401">

</xml_diff>

<commit_message>
Add generated leaderboard data - 2024-04-14T23:06:15
</commit_message>
<xml_diff>
--- a/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
+++ b/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
@@ -128,6 +128,18 @@
     <t>54.47%</t>
   </si>
   <si>
+    <t>22R01A05Q2</t>
+  </si>
+  <si>
+    <t>22r01a05q2</t>
+  </si>
+  <si>
+    <t>praneetha5q2</t>
+  </si>
+  <si>
+    <t>50.48%</t>
+  </si>
+  <si>
     <t>22R01A0531</t>
   </si>
   <si>
@@ -158,18 +170,6 @@
     <t>49.83%</t>
   </si>
   <si>
-    <t>22R01A05Q2</t>
-  </si>
-  <si>
-    <t>22r01a05q2</t>
-  </si>
-  <si>
-    <t>praneetha5q2</t>
-  </si>
-  <si>
-    <t>48.52%</t>
-  </si>
-  <si>
     <t>22R01A0597</t>
   </si>
   <si>
@@ -206,6 +206,21 @@
     <t>48.28%</t>
   </si>
   <si>
+    <t>22R01A05N4</t>
+  </si>
+  <si>
+    <t>mkeerthi63027</t>
+  </si>
+  <si>
+    <t>mkeerthify</t>
+  </si>
+  <si>
+    <t>keerthi_mangali</t>
+  </si>
+  <si>
+    <t>48.03%</t>
+  </si>
+  <si>
     <t>22R01A05B2</t>
   </si>
   <si>
@@ -221,21 +236,6 @@
     <t>47.96%</t>
   </si>
   <si>
-    <t>22R01A05N4</t>
-  </si>
-  <si>
-    <t>mkeerthi63027</t>
-  </si>
-  <si>
-    <t>mkeerthify</t>
-  </si>
-  <si>
-    <t>keerthi_mangali</t>
-  </si>
-  <si>
-    <t>46.67%</t>
-  </si>
-  <si>
     <t>22R01A05A1</t>
   </si>
   <si>
@@ -353,7 +353,7 @@
     <t>@KIREET_5L5</t>
   </si>
   <si>
-    <t>42.43%</t>
+    <t>42.45%</t>
   </si>
   <si>
     <t>22R01A73B1</t>
@@ -716,7 +716,7 @@
     <t>@msaiteja665</t>
   </si>
   <si>
-    <t>34.35%</t>
+    <t>34.37%</t>
   </si>
   <si>
     <t>22R01A67D1</t>
@@ -950,7 +950,7 @@
     <t>cmr_22r01a73b6</t>
   </si>
   <si>
-    <t>28.91%</t>
+    <t>28.95%</t>
   </si>
   <si>
     <t>22R01A0552</t>
@@ -10069,13 +10069,13 @@
         <v>39</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>779.0</v>
+        <v>816.0</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>39</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>60.0</v>
+        <v>0.0</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>0.0</v>
@@ -10084,19 +10084,19 @@
         <v>39</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>1349.0</v>
+        <v>1490.0</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>40</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>1413.0</v>
+        <v>1050.0</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>39</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>6.0</v>
+        <v>156.0</v>
       </c>
       <c r="N8" s="2" t="s">
         <v>41</v>
@@ -10113,37 +10113,37 @@
         <v>43</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>624.0</v>
+        <v>779.0</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>60.0</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>1349.0</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F9" s="2" t="n">
-        <v>94.0</v>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>72.0</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="I9" s="2" t="n">
-        <v>1409.0</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>46</v>
-      </c>
       <c r="K9" s="2" t="n">
-        <v>1320.0</v>
+        <v>1413.0</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>43</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>4.0</v>
+        <v>6.0</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
@@ -10151,40 +10151,40 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>624.0</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>753.0</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="F10" s="2" t="n">
-        <v>0.0</v>
+        <v>94.0</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.0</v>
+        <v>72.0</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>49</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>1490.0</v>
+        <v>1409.0</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>50</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>1050.0</v>
+        <v>1320.0</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>156.0</v>
+        <v>4.0</v>
       </c>
       <c r="N10" s="2" t="s">
         <v>51</v>
@@ -10289,7 +10289,7 @@
         <v>65</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>807.0</v>
+        <v>755.0</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>66</v>
@@ -10301,22 +10301,22 @@
         <v>0.0</v>
       </c>
       <c r="H13" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>1477.0</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="I13" s="2" t="n">
-        <v>1424.0</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="K13" s="2" t="n">
-        <v>1139.0</v>
+        <v>1092.0</v>
       </c>
       <c r="L13" s="2" t="s">
         <v>65</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>114.0</v>
+        <v>143.0</v>
       </c>
       <c r="N13" s="2" t="s">
         <v>68</v>
@@ -10333,7 +10333,7 @@
         <v>70</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>711.0</v>
+        <v>807.0</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>71</v>
@@ -10345,22 +10345,22 @@
         <v>0.0</v>
       </c>
       <c r="H14" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>1424.0</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="I14" s="2" t="n">
-        <v>1477.0</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="K14" s="2" t="n">
-        <v>1092.0</v>
+        <v>1139.0</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>70</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>143.0</v>
+        <v>114.0</v>
       </c>
       <c r="N14" s="2" t="s">
         <v>73</v>
@@ -10650,7 +10650,7 @@
         <v>40.0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>127.0</v>
+        <v>129.0</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>110</v>
@@ -11706,7 +11706,7 @@
         <v>118.0</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>116.0</v>
+        <v>118.0</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>231</v>
@@ -12454,7 +12454,7 @@
         <v>10.0</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>64.0</v>
+        <v>68.0</v>
       </c>
       <c r="H62" s="2" t="s">
         <v>310</v>

</xml_diff>

<commit_message>
Add generated leaderboard data - 2024-04-18T19:07:30
</commit_message>
<xml_diff>
--- a/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
+++ b/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
@@ -233,6 +233,24 @@
     <t>keerthi_mangali</t>
   </si>
   <si>
+    <t>22R01A66A5</t>
+  </si>
+  <si>
+    <t>22r01a66a5</t>
+  </si>
+  <si>
+    <t>22r01a9x5i</t>
+  </si>
+  <si>
+    <t>shivakrishna21</t>
+  </si>
+  <si>
+    <t>shivakrishnamur1</t>
+  </si>
+  <si>
+    <t>47.32%</t>
+  </si>
+  <si>
     <t>22R01A05A1</t>
   </si>
   <si>
@@ -264,24 +282,6 @@
   </si>
   <si>
     <t>45.26%</t>
-  </si>
-  <si>
-    <t>22R01A66A5</t>
-  </si>
-  <si>
-    <t>22r01a66a5</t>
-  </si>
-  <si>
-    <t>22r01a9x5i</t>
-  </si>
-  <si>
-    <t>shivakrishna21</t>
-  </si>
-  <si>
-    <t>shivakrishnamur1</t>
-  </si>
-  <si>
-    <t>44.75%</t>
   </si>
   <si>
     <t>22R01A66D1</t>
@@ -10386,34 +10386,34 @@
         <v>74</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>895.0</v>
+        <v>709.0</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>75</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.0</v>
+        <v>37.0</v>
       </c>
       <c r="H15" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>1511.0</v>
+      </c>
+      <c r="J15" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="I15" s="2" t="n">
-        <v>1475.0</v>
-      </c>
-      <c r="J15" s="2" t="s">
+      <c r="K15" s="2" t="n">
+        <v>1544.0</v>
+      </c>
+      <c r="L15" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="K15" s="2" t="n">
-        <v>1411.0</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="M15" s="2" t="n">
-        <v>1.0</v>
+        <v>74.0</v>
       </c>
       <c r="N15" s="2" t="s">
         <v>78</v>
@@ -10430,7 +10430,7 @@
         <v>80</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>760.0</v>
+        <v>895.0</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>81</v>
@@ -10442,25 +10442,25 @@
         <v>0.0</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>1434.0</v>
+        <v>1475.0</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>1054.0</v>
+        <v>1411.0</v>
       </c>
       <c r="L16" s="2" t="s">
         <v>80</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>103.0</v>
+        <v>1.0</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17">
@@ -10468,40 +10468,40 @@
         <v>16.0</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>709.0</v>
+        <v>760.0</v>
       </c>
       <c r="E17" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H17" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="F17" s="2" t="n">
-        <v>10.0</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>37.0</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>84</v>
-      </c>
       <c r="I17" s="2" t="n">
-        <v>1511.0</v>
+        <v>1434.0</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>1544.0</v>
+        <v>1054.0</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>29.0</v>
+        <v>103.0</v>
       </c>
       <c r="N17" s="2" t="s">
         <v>89</v>

</xml_diff>

<commit_message>
Add generated leaderboard data - 2024-04-20T19:07:23
</commit_message>
<xml_diff>
--- a/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
+++ b/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
@@ -221,7 +221,7 @@
     <t>22r01a05l1</t>
   </si>
   <si>
-    <t>48.17%</t>
+    <t>48.21%</t>
   </si>
   <si>
     <t>22R01A05B2</t>
@@ -341,7 +341,7 @@
     <t>@KIREET_5L5</t>
   </si>
   <si>
-    <t>42.42%</t>
+    <t>42.44%</t>
   </si>
   <si>
     <t>22R01A66B1</t>
@@ -416,7 +416,7 @@
     <t>macom_harshita</t>
   </si>
   <si>
-    <t>41.01%</t>
+    <t>41.26%</t>
   </si>
   <si>
     <t>22R01A66E8</t>
@@ -10298,7 +10298,7 @@
         <v>40.0</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>102.0</v>
+        <v>106.0</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>66</v>
@@ -10606,7 +10606,7 @@
         <v>40.0</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>137.0</v>
+        <v>139.0</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>106</v>
@@ -10844,7 +10844,7 @@
         <v>133</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>36.0</v>
+        <v>41.0</v>
       </c>
       <c r="N25" s="2" t="s">
         <v>134</v>

</xml_diff>

<commit_message>
Add generated leaderboard data - 2024-04-26T19:07:54
</commit_message>
<xml_diff>
--- a/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
+++ b/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
@@ -143,7 +143,7 @@
     <t>shivakrishnamur1</t>
   </si>
   <si>
-    <t>53.03%</t>
+    <t>53.26%</t>
   </si>
   <si>
     <t>22R01A05L1</t>
@@ -164,7 +164,7 @@
     <t>22r01a05l1</t>
   </si>
   <si>
-    <t>51.37%</t>
+    <t>51.39%</t>
   </si>
   <si>
     <t>22R01A05Q6</t>
@@ -242,7 +242,7 @@
     <t>@KIREET_5L5</t>
   </si>
   <si>
-    <t>48.11%</t>
+    <t>48.13%</t>
   </si>
   <si>
     <t>22R01A05B2</t>
@@ -638,7 +638,7 @@
     <t>eshu5886</t>
   </si>
   <si>
-    <t>35.92%</t>
+    <t>35.93%</t>
   </si>
   <si>
     <t>22R01A66F7</t>
@@ -713,7 +713,7 @@
     <t>@msaiteja665</t>
   </si>
   <si>
-    <t>34.44%</t>
+    <t>34.46%</t>
   </si>
   <si>
     <t>22R01A67D1</t>
@@ -10222,7 +10222,7 @@
         <v>10.0</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>41.0</v>
+        <v>65.0</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>38</v>
@@ -10266,7 +10266,7 @@
         <v>40.0</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>166.0</v>
+        <v>168.0</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>47</v>
@@ -10486,7 +10486,7 @@
         <v>40.0</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>177.0</v>
+        <v>179.0</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>73</v>
@@ -11674,7 +11674,7 @@
         <v>17.0</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>8.0</v>
+        <v>10.0</v>
       </c>
       <c r="H41" s="2" t="s">
         <v>206</v>
@@ -11850,7 +11850,7 @@
         <v>118.0</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>128.0</v>
+        <v>130.0</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>230</v>

</xml_diff>

<commit_message>
Add generated leaderboard data - 2024-04-27T19:07:42
</commit_message>
<xml_diff>
--- a/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
+++ b/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
@@ -164,7 +164,7 @@
     <t>22r01a05l1</t>
   </si>
   <si>
-    <t>51.39%</t>
+    <t>51.51%</t>
   </si>
   <si>
     <t>22R01A05Q6</t>
@@ -242,7 +242,7 @@
     <t>@KIREET_5L5</t>
   </si>
   <si>
-    <t>48.13%</t>
+    <t>48.24%</t>
   </si>
   <si>
     <t>22R01A05B2</t>
@@ -1445,7 +1445,7 @@
     <t>cmr_22r01a0560</t>
   </si>
   <si>
-    <t>26.15%</t>
+    <t>26.17%</t>
   </si>
   <si>
     <t>22R01A05D6</t>
@@ -10266,7 +10266,7 @@
         <v>40.0</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>168.0</v>
+        <v>180.0</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>47</v>
@@ -10486,7 +10486,7 @@
         <v>40.0</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>179.0</v>
+        <v>191.0</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>73</v>
@@ -14138,7 +14138,7 @@
         <v>0.0</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>0.0</v>
+        <v>3.0</v>
       </c>
       <c r="H97" s="2" t="s">
         <v>474</v>

</xml_diff>

<commit_message>
Add generated leaderboard data - 2024-05-05T19:07:26
</commit_message>
<xml_diff>
--- a/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
+++ b/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
@@ -113,6 +113,27 @@
     <t>55.56%</t>
   </si>
   <si>
+    <t>22R01A05L1</t>
+  </si>
+  <si>
+    <t>bobbalavarshithreddy</t>
+  </si>
+  <si>
+    <t>22r01aupp6</t>
+  </si>
+  <si>
+    <t>varshith__reddie</t>
+  </si>
+  <si>
+    <t>v22r01a05l1</t>
+  </si>
+  <si>
+    <t>22r01a05l1</t>
+  </si>
+  <si>
+    <t>55.22%</t>
+  </si>
+  <si>
     <t>22R01A05Q6</t>
   </si>
   <si>
@@ -146,27 +167,6 @@
     <t>53.32%</t>
   </si>
   <si>
-    <t>22R01A05L1</t>
-  </si>
-  <si>
-    <t>bobbalavarshithreddy</t>
-  </si>
-  <si>
-    <t>22r01aupp6</t>
-  </si>
-  <si>
-    <t>varshith__reddie</t>
-  </si>
-  <si>
-    <t>v22r01a05l1</t>
-  </si>
-  <si>
-    <t>22r01a05l1</t>
-  </si>
-  <si>
-    <t>52.76%</t>
-  </si>
-  <si>
     <t>22R01A66A5</t>
   </si>
   <si>
@@ -1724,6 +1724,15 @@
     <t>25.76%</t>
   </si>
   <si>
+    <t>22R01A6670</t>
+  </si>
+  <si>
+    <t>varshini_arige</t>
+  </si>
+  <si>
+    <t>25.71%</t>
+  </si>
+  <si>
     <t>22R01A6667</t>
   </si>
   <si>
@@ -1892,15 +1901,6 @@
     <t>24.48%</t>
   </si>
   <si>
-    <t>22R01A6670</t>
-  </si>
-  <si>
-    <t>varshini_arige</t>
-  </si>
-  <si>
-    <t>24.44%</t>
-  </si>
-  <si>
     <t>22R01A7355</t>
   </si>
   <si>
@@ -4079,6 +4079,21 @@
     <t>7.64%</t>
   </si>
   <si>
+    <t>22R01A66A2</t>
+  </si>
+  <si>
+    <t>22r01a66a2</t>
+  </si>
+  <si>
+    <t>22r01az40l</t>
+  </si>
+  <si>
+    <t>a22r01a66a2</t>
+  </si>
+  <si>
+    <t>7.63%</t>
+  </si>
+  <si>
     <t>22R01A7331</t>
   </si>
   <si>
@@ -4953,21 +4968,6 @@
   </si>
   <si>
     <t>6.29%</t>
-  </si>
-  <si>
-    <t>22R01A66A2</t>
-  </si>
-  <si>
-    <t>22r01a66a2</t>
-  </si>
-  <si>
-    <t>22r01az40l</t>
-  </si>
-  <si>
-    <t>a22r01a66a2</t>
-  </si>
-  <si>
-    <t>6.28%</t>
   </si>
   <si>
     <t>22R01A04H1</t>
@@ -10550,37 +10550,37 @@
         <v>34</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>775.0</v>
+        <v>904.0</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>35</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>104.0</v>
+        <v>70.0</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>102.0</v>
+        <v>200.0</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>36</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>1371.0</v>
+        <v>1394.0</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>37</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>1376.0</v>
+        <v>1371.0</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8">
@@ -10588,43 +10588,43 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>779.0</v>
+        <v>775.0</v>
       </c>
       <c r="E8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>104.0</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>102.0</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>1371.0</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>1376.0</v>
+      </c>
+      <c r="L8" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="2" t="n">
-        <v>93.0</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>19.0</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>1575.0</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="K8" s="2" t="n">
-        <v>1320.0</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="M8" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9">
@@ -10632,34 +10632,34 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>904.0</v>
+        <v>779.0</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>50.0</v>
+        <v>93.0</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>200.0</v>
+        <v>19.0</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>47</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>1394.0</v>
+        <v>1575.0</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>1371.0</v>
+        <v>1320.0</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>49</v>
@@ -15390,16 +15390,16 @@
         <v>571</v>
       </c>
       <c r="D117" s="2" t="n">
-        <v>608.0</v>
+        <v>614.0</v>
       </c>
       <c r="E117" s="2" t="s">
         <v>571</v>
       </c>
       <c r="F117" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="G117" s="2" t="n">
-        <v>50.0</v>
+        <v>4.0</v>
       </c>
       <c r="H117" s="2" t="s">
         <v>571</v>
@@ -15411,16 +15411,16 @@
         <v>571</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>1050.0</v>
+        <v>932.0</v>
       </c>
       <c r="L117" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="M117" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N117" s="2" t="s">
         <v>572</v>
-      </c>
-      <c r="M117" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N117" s="2" t="s">
-        <v>573</v>
       </c>
     </row>
     <row r="118">
@@ -15428,43 +15428,43 @@
         <v>117.0</v>
       </c>
       <c r="B118" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="C118" s="2" t="s">
         <v>574</v>
       </c>
-      <c r="C118" s="2" t="s">
+      <c r="D118" s="2" t="n">
+        <v>608.0</v>
+      </c>
+      <c r="E118" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="F118" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G118" s="2" t="n">
+        <v>50.0</v>
+      </c>
+      <c r="H118" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="I118" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J118" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="K118" s="2" t="n">
+        <v>1050.0</v>
+      </c>
+      <c r="L118" s="2" t="s">
         <v>575</v>
       </c>
-      <c r="D118" s="2" t="n">
-        <v>354.0</v>
-      </c>
-      <c r="E118" s="2" t="s">
-        <v>575</v>
-      </c>
-      <c r="F118" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G118" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H118" s="2" t="s">
-        <v>575</v>
-      </c>
-      <c r="I118" s="2" t="n">
-        <v>1438.0</v>
-      </c>
-      <c r="J118" s="2" t="s">
-        <v>575</v>
-      </c>
-      <c r="K118" s="2" t="n">
-        <v>887.0</v>
-      </c>
-      <c r="L118" s="2" t="s">
+      <c r="M118" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N118" s="2" t="s">
         <v>576</v>
-      </c>
-      <c r="M118" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N118" s="2" t="s">
-        <v>577</v>
       </c>
     </row>
     <row r="119">
@@ -15472,16 +15472,16 @@
         <v>118.0</v>
       </c>
       <c r="B119" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="C119" s="2" t="s">
         <v>578</v>
       </c>
-      <c r="C119" s="2" t="s">
-        <v>579</v>
-      </c>
       <c r="D119" s="2" t="n">
-        <v>635.0</v>
+        <v>354.0</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>201</v>
+        <v>578</v>
       </c>
       <c r="F119" s="2" t="n">
         <v>0.0</v>
@@ -15493,22 +15493,22 @@
         <v>578</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>0.0</v>
+        <v>1438.0</v>
       </c>
       <c r="J119" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="K119" s="2" t="n">
+        <v>887.0</v>
+      </c>
+      <c r="L119" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="M119" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N119" s="2" t="s">
         <v>580</v>
-      </c>
-      <c r="K119" s="2" t="n">
-        <v>864.0</v>
-      </c>
-      <c r="L119" s="2" t="s">
-        <v>581</v>
-      </c>
-      <c r="M119" s="2" t="n">
-        <v>12.0</v>
-      </c>
-      <c r="N119" s="2" t="s">
-        <v>582</v>
       </c>
     </row>
     <row r="120">
@@ -15516,43 +15516,43 @@
         <v>119.0</v>
       </c>
       <c r="B120" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="D120" s="2" t="n">
+        <v>635.0</v>
+      </c>
+      <c r="E120" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F120" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G120" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H120" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="I120" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J120" s="2" t="s">
         <v>583</v>
       </c>
-      <c r="C120" s="2" t="s">
+      <c r="K120" s="2" t="n">
+        <v>864.0</v>
+      </c>
+      <c r="L120" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="D120" s="2" t="n">
-        <v>345.0</v>
-      </c>
-      <c r="E120" s="2" t="s">
+      <c r="M120" s="2" t="n">
+        <v>12.0</v>
+      </c>
+      <c r="N120" s="2" t="s">
         <v>585</v>
-      </c>
-      <c r="F120" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G120" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H120" s="2" t="s">
-        <v>586</v>
-      </c>
-      <c r="I120" s="2" t="n">
-        <v>1422.0</v>
-      </c>
-      <c r="J120" s="2" t="s">
-        <v>586</v>
-      </c>
-      <c r="K120" s="2" t="n">
-        <v>925.0</v>
-      </c>
-      <c r="L120" s="2" t="s">
-        <v>587</v>
-      </c>
-      <c r="M120" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N120" s="2" t="s">
-        <v>588</v>
       </c>
     </row>
     <row r="121">
@@ -15560,34 +15560,34 @@
         <v>120.0</v>
       </c>
       <c r="B121" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="D121" s="2" t="n">
+        <v>345.0</v>
+      </c>
+      <c r="E121" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="F121" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G121" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H121" s="2" t="s">
         <v>589</v>
       </c>
-      <c r="C121" s="2" t="s">
-        <v>590</v>
-      </c>
-      <c r="D121" s="2" t="n">
-        <v>357.0</v>
-      </c>
-      <c r="E121" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F121" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G121" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H121" s="2" t="s">
-        <v>590</v>
-      </c>
       <c r="I121" s="2" t="n">
-        <v>1410.0</v>
+        <v>1422.0</v>
       </c>
       <c r="J121" s="2" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>865.0</v>
+        <v>925.0</v>
       </c>
       <c r="L121" s="2" t="s">
         <v>590</v>
@@ -15596,7 +15596,7 @@
         <v>0.0</v>
       </c>
       <c r="N121" s="2" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="122">
@@ -15604,43 +15604,43 @@
         <v>121.0</v>
       </c>
       <c r="B122" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="C122" s="2" t="s">
         <v>593</v>
       </c>
-      <c r="C122" s="2" t="s">
+      <c r="D122" s="2" t="n">
+        <v>357.0</v>
+      </c>
+      <c r="E122" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F122" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G122" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H122" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="I122" s="2" t="n">
+        <v>1410.0</v>
+      </c>
+      <c r="J122" s="2" t="s">
         <v>594</v>
       </c>
-      <c r="D122" s="2" t="n">
-        <v>611.0</v>
-      </c>
-      <c r="E122" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F122" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G122" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H122" s="2" t="s">
-        <v>594</v>
-      </c>
-      <c r="I122" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J122" s="2" t="s">
+      <c r="K122" s="2" t="n">
+        <v>865.0</v>
+      </c>
+      <c r="L122" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="M122" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N122" s="2" t="s">
         <v>595</v>
-      </c>
-      <c r="K122" s="2" t="n">
-        <v>1006.0</v>
-      </c>
-      <c r="L122" s="2" t="s">
-        <v>596</v>
-      </c>
-      <c r="M122" s="2" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="N122" s="2" t="s">
-        <v>597</v>
       </c>
     </row>
     <row r="123">
@@ -15648,43 +15648,43 @@
         <v>122.0</v>
       </c>
       <c r="B123" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="D123" s="2" t="n">
+        <v>611.0</v>
+      </c>
+      <c r="E123" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F123" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G123" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H123" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="I123" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J123" s="2" t="s">
         <v>598</v>
       </c>
-      <c r="C123" s="2" t="s">
-        <v>599</v>
-      </c>
-      <c r="D123" s="2" t="n">
-        <v>587.0</v>
-      </c>
-      <c r="E123" s="2" t="s">
-        <v>599</v>
-      </c>
-      <c r="F123" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G123" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H123" s="2" t="s">
-        <v>599</v>
-      </c>
-      <c r="I123" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J123" s="2" t="s">
-        <v>600</v>
-      </c>
       <c r="K123" s="2" t="n">
-        <v>1002.0</v>
+        <v>1006.0</v>
       </c>
       <c r="L123" s="2" t="s">
         <v>599</v>
       </c>
       <c r="M123" s="2" t="n">
-        <v>15.0</v>
+        <v>4.0</v>
       </c>
       <c r="N123" s="2" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
     </row>
     <row r="124">
@@ -15692,16 +15692,16 @@
         <v>123.0</v>
       </c>
       <c r="B124" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="C124" s="2" t="s">
         <v>602</v>
       </c>
-      <c r="C124" s="2" t="s">
-        <v>603</v>
-      </c>
       <c r="D124" s="2" t="n">
-        <v>584.0</v>
+        <v>587.0</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="F124" s="2" t="n">
         <v>0.0</v>
@@ -15710,7 +15710,7 @@
         <v>0.0</v>
       </c>
       <c r="H124" s="2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="I124" s="2" t="n">
         <v>0.0</v>
@@ -15719,16 +15719,16 @@
         <v>603</v>
       </c>
       <c r="K124" s="2" t="n">
-        <v>1130.0</v>
+        <v>1002.0</v>
       </c>
       <c r="L124" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="M124" s="2" t="n">
+        <v>15.0</v>
+      </c>
+      <c r="N124" s="2" t="s">
         <v>604</v>
-      </c>
-      <c r="M124" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N124" s="2" t="s">
-        <v>605</v>
       </c>
     </row>
     <row r="125">
@@ -15736,43 +15736,43 @@
         <v>124.0</v>
       </c>
       <c r="B125" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="C125" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="C125" s="2" t="s">
+      <c r="D125" s="2" t="n">
+        <v>584.0</v>
+      </c>
+      <c r="E125" s="2" t="s">
+        <v>606</v>
+      </c>
+      <c r="F125" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G125" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H125" s="2" t="s">
+        <v>606</v>
+      </c>
+      <c r="I125" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J125" s="2" t="s">
+        <v>606</v>
+      </c>
+      <c r="K125" s="2" t="n">
+        <v>1130.0</v>
+      </c>
+      <c r="L125" s="2" t="s">
         <v>607</v>
       </c>
-      <c r="D125" s="2" t="n">
-        <v>595.0</v>
-      </c>
-      <c r="E125" s="2" t="s">
+      <c r="M125" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N125" s="2" t="s">
         <v>608</v>
-      </c>
-      <c r="F125" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G125" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H125" s="2" t="s">
-        <v>609</v>
-      </c>
-      <c r="I125" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J125" s="2" t="s">
-        <v>609</v>
-      </c>
-      <c r="K125" s="2" t="n">
-        <v>1059.0</v>
-      </c>
-      <c r="L125" s="2" t="s">
-        <v>610</v>
-      </c>
-      <c r="M125" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N125" s="2" t="s">
-        <v>611</v>
       </c>
     </row>
     <row r="126">
@@ -15780,43 +15780,43 @@
         <v>125.0</v>
       </c>
       <c r="B126" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="D126" s="2" t="n">
+        <v>595.0</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="F126" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G126" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H126" s="2" t="s">
         <v>612</v>
       </c>
-      <c r="C126" s="2" t="s">
+      <c r="I126" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J126" s="2" t="s">
+        <v>612</v>
+      </c>
+      <c r="K126" s="2" t="n">
+        <v>1059.0</v>
+      </c>
+      <c r="L126" s="2" t="s">
         <v>613</v>
       </c>
-      <c r="D126" s="2" t="n">
-        <v>598.0</v>
-      </c>
-      <c r="E126" s="2" t="s">
+      <c r="M126" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N126" s="2" t="s">
         <v>614</v>
-      </c>
-      <c r="F126" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G126" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H126" s="2" t="s">
-        <v>615</v>
-      </c>
-      <c r="I126" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J126" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="K126" s="2" t="n">
-        <v>1036.0</v>
-      </c>
-      <c r="L126" s="2" t="s">
-        <v>617</v>
-      </c>
-      <c r="M126" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N126" s="2" t="s">
-        <v>618</v>
       </c>
     </row>
     <row r="127">
@@ -15824,43 +15824,43 @@
         <v>126.0</v>
       </c>
       <c r="B127" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="D127" s="2" t="n">
+        <v>598.0</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="F127" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G127" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H127" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="I127" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J127" s="2" t="s">
         <v>619</v>
       </c>
-      <c r="C127" s="2" t="s">
+      <c r="K127" s="2" t="n">
+        <v>1036.0</v>
+      </c>
+      <c r="L127" s="2" t="s">
         <v>620</v>
       </c>
-      <c r="D127" s="2" t="n">
-        <v>589.0</v>
-      </c>
-      <c r="E127" s="2" t="s">
+      <c r="M127" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N127" s="2" t="s">
         <v>621</v>
-      </c>
-      <c r="F127" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G127" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H127" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="I127" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J127" s="2" t="s">
-        <v>623</v>
-      </c>
-      <c r="K127" s="2" t="n">
-        <v>1053.0</v>
-      </c>
-      <c r="L127" s="2" t="s">
-        <v>624</v>
-      </c>
-      <c r="M127" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N127" s="2" t="s">
-        <v>625</v>
       </c>
     </row>
     <row r="128">
@@ -15868,34 +15868,34 @@
         <v>127.0</v>
       </c>
       <c r="B128" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="D128" s="2" t="n">
+        <v>589.0</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="F128" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G128" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H128" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="I128" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J128" s="2" t="s">
         <v>626</v>
       </c>
-      <c r="C128" s="2" t="s">
-        <v>627</v>
-      </c>
-      <c r="D128" s="2" t="n">
-        <v>614.0</v>
-      </c>
-      <c r="E128" s="2" t="s">
-        <v>627</v>
-      </c>
-      <c r="F128" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G128" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H128" s="2" t="s">
-        <v>627</v>
-      </c>
-      <c r="I128" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J128" s="2" t="s">
-        <v>627</v>
-      </c>
       <c r="K128" s="2" t="n">
-        <v>932.0</v>
+        <v>1053.0</v>
       </c>
       <c r="L128" s="2" t="s">
         <v>627</v>
@@ -22433,13 +22433,13 @@
         <v>0.0</v>
       </c>
       <c r="E277" s="2" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="F277" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G277" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="H277" s="2" t="s">
         <v>1356</v>
@@ -22448,19 +22448,19 @@
         <v>0.0</v>
       </c>
       <c r="J277" s="2" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="K277" s="2" t="n">
-        <v>1179.0</v>
+        <v>926.0</v>
       </c>
       <c r="L277" s="2" t="s">
         <v>1356</v>
       </c>
       <c r="M277" s="2" t="n">
-        <v>0.0</v>
+        <v>31.0</v>
       </c>
       <c r="N277" s="2" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="278">
@@ -22468,16 +22468,16 @@
         <v>277.0</v>
       </c>
       <c r="B278" s="2" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="D278" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E278" s="2" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="F278" s="2" t="n">
         <v>0.0</v>
@@ -22486,25 +22486,25 @@
         <v>0.0</v>
       </c>
       <c r="H278" s="2" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="I278" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J278" s="2" t="s">
+        <v>1362</v>
+      </c>
+      <c r="K278" s="2" t="n">
+        <v>1179.0</v>
+      </c>
+      <c r="L278" s="2" t="s">
         <v>1361</v>
       </c>
-      <c r="K278" s="2" t="n">
-        <v>1166.0</v>
-      </c>
-      <c r="L278" s="2" t="s">
-        <v>1360</v>
-      </c>
       <c r="M278" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N278" s="2" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
     </row>
     <row r="279">
@@ -22512,16 +22512,16 @@
         <v>278.0</v>
       </c>
       <c r="B279" s="2" t="s">
-        <v>1363</v>
+        <v>1364</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>1363</v>
+        <v>1365</v>
       </c>
       <c r="D279" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E279" s="2" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="F279" s="2" t="n">
         <v>0.0</v>
@@ -22536,13 +22536,13 @@
         <v>0.0</v>
       </c>
       <c r="J279" s="2" t="s">
+        <v>1366</v>
+      </c>
+      <c r="K279" s="2" t="n">
+        <v>1166.0</v>
+      </c>
+      <c r="L279" s="2" t="s">
         <v>1365</v>
-      </c>
-      <c r="K279" s="2" t="n">
-        <v>1161.0</v>
-      </c>
-      <c r="L279" s="2" t="s">
-        <v>1366</v>
       </c>
       <c r="M279" s="2" t="n">
         <v>0.0</v>
@@ -22559,7 +22559,7 @@
         <v>1368</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>1369</v>
+        <v>1368</v>
       </c>
       <c r="D280" s="2" t="n">
         <v>0.0</v>
@@ -22574,7 +22574,7 @@
         <v>0.0</v>
       </c>
       <c r="H280" s="2" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="I280" s="2" t="n">
         <v>0.0</v>
@@ -22583,16 +22583,16 @@
         <v>1370</v>
       </c>
       <c r="K280" s="2" t="n">
-        <v>971.0</v>
+        <v>1161.0</v>
       </c>
       <c r="L280" s="2" t="s">
-        <v>1369</v>
+        <v>1371</v>
       </c>
       <c r="M280" s="2" t="n">
-        <v>24.0</v>
+        <v>0.0</v>
       </c>
       <c r="N280" s="2" t="s">
-        <v>1371</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="281">
@@ -22600,16 +22600,16 @@
         <v>280.0</v>
       </c>
       <c r="B281" s="2" t="s">
-        <v>1372</v>
+        <v>1373</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>1373</v>
+        <v>1374</v>
       </c>
       <c r="D281" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E281" s="2" t="s">
-        <v>201</v>
+        <v>1374</v>
       </c>
       <c r="F281" s="2" t="n">
         <v>0.0</v>
@@ -22618,25 +22618,25 @@
         <v>0.0</v>
       </c>
       <c r="H281" s="2" t="s">
-        <v>201</v>
+        <v>1374</v>
       </c>
       <c r="I281" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J281" s="2" t="s">
+        <v>1375</v>
+      </c>
+      <c r="K281" s="2" t="n">
+        <v>971.0</v>
+      </c>
+      <c r="L281" s="2" t="s">
         <v>1374</v>
       </c>
-      <c r="K281" s="2" t="n">
-        <v>1146.0</v>
-      </c>
-      <c r="L281" s="2" t="s">
-        <v>1373</v>
-      </c>
       <c r="M281" s="2" t="n">
-        <v>0.0</v>
+        <v>24.0</v>
       </c>
       <c r="N281" s="2" t="s">
-        <v>1375</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="282">
@@ -22644,10 +22644,10 @@
         <v>281.0</v>
       </c>
       <c r="B282" s="2" t="s">
-        <v>1376</v>
+        <v>1377</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>1377</v>
+        <v>1378</v>
       </c>
       <c r="D282" s="2" t="n">
         <v>0.0</v>
@@ -22662,7 +22662,7 @@
         <v>0.0</v>
       </c>
       <c r="H282" s="2" t="s">
-        <v>1378</v>
+        <v>201</v>
       </c>
       <c r="I282" s="2" t="n">
         <v>0.0</v>
@@ -22671,16 +22671,16 @@
         <v>1379</v>
       </c>
       <c r="K282" s="2" t="n">
-        <v>1141.0</v>
+        <v>1146.0</v>
       </c>
       <c r="L282" s="2" t="s">
+        <v>1378</v>
+      </c>
+      <c r="M282" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N282" s="2" t="s">
         <v>1380</v>
-      </c>
-      <c r="M282" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N282" s="2" t="s">
-        <v>1381</v>
       </c>
     </row>
     <row r="283">
@@ -22688,43 +22688,43 @@
         <v>282.0</v>
       </c>
       <c r="B283" s="2" t="s">
+        <v>1381</v>
+      </c>
+      <c r="C283" s="2" t="s">
         <v>1382</v>
       </c>
-      <c r="C283" s="2" t="s">
-        <v>201</v>
-      </c>
       <c r="D283" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E283" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F283" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G283" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H283" s="2" t="s">
         <v>1383</v>
       </c>
-      <c r="F283" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G283" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H283" s="2" t="s">
+      <c r="I283" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J283" s="2" t="s">
         <v>1384</v>
-      </c>
-      <c r="I283" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J283" s="2" t="s">
-        <v>1385</v>
       </c>
       <c r="K283" s="2" t="n">
         <v>1141.0</v>
       </c>
       <c r="L283" s="2" t="s">
+        <v>1385</v>
+      </c>
+      <c r="M283" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N283" s="2" t="s">
         <v>1386</v>
-      </c>
-      <c r="M283" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N283" s="2" t="s">
-        <v>1381</v>
       </c>
     </row>
     <row r="284">
@@ -22741,7 +22741,7 @@
         <v>0.0</v>
       </c>
       <c r="E284" s="2" t="s">
-        <v>201</v>
+        <v>1388</v>
       </c>
       <c r="F284" s="2" t="n">
         <v>0.0</v>
@@ -22750,25 +22750,25 @@
         <v>0.0</v>
       </c>
       <c r="H284" s="2" t="s">
-        <v>1388</v>
+        <v>1389</v>
       </c>
       <c r="I284" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J284" s="2" t="s">
-        <v>1389</v>
+        <v>1390</v>
       </c>
       <c r="K284" s="2" t="n">
-        <v>921.0</v>
+        <v>1141.0</v>
       </c>
       <c r="L284" s="2" t="s">
-        <v>1390</v>
+        <v>1391</v>
       </c>
       <c r="M284" s="2" t="n">
-        <v>28.0</v>
+        <v>0.0</v>
       </c>
       <c r="N284" s="2" t="s">
-        <v>1391</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="285">
@@ -22785,16 +22785,16 @@
         <v>0.0</v>
       </c>
       <c r="E285" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F285" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G285" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H285" s="2" t="s">
         <v>1393</v>
-      </c>
-      <c r="F285" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G285" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H285" s="2" t="s">
-        <v>201</v>
       </c>
       <c r="I285" s="2" t="n">
         <v>0.0</v>
@@ -22803,16 +22803,16 @@
         <v>1394</v>
       </c>
       <c r="K285" s="2" t="n">
-        <v>1134.0</v>
+        <v>921.0</v>
       </c>
       <c r="L285" s="2" t="s">
-        <v>201</v>
+        <v>1395</v>
       </c>
       <c r="M285" s="2" t="n">
-        <v>0.0</v>
+        <v>28.0</v>
       </c>
       <c r="N285" s="2" t="s">
-        <v>1395</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="286">
@@ -22820,16 +22820,16 @@
         <v>285.0</v>
       </c>
       <c r="B286" s="2" t="s">
-        <v>1396</v>
+        <v>1397</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>1396</v>
+        <v>201</v>
       </c>
       <c r="D286" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E286" s="2" t="s">
-        <v>1397</v>
+        <v>1398</v>
       </c>
       <c r="F286" s="2" t="n">
         <v>0.0</v>
@@ -22838,19 +22838,19 @@
         <v>0.0</v>
       </c>
       <c r="H286" s="2" t="s">
-        <v>1396</v>
+        <v>201</v>
       </c>
       <c r="I286" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J286" s="2" t="s">
-        <v>1398</v>
+        <v>1399</v>
       </c>
       <c r="K286" s="2" t="n">
-        <v>1132.0</v>
+        <v>1134.0</v>
       </c>
       <c r="L286" s="2" t="s">
-        <v>1399</v>
+        <v>201</v>
       </c>
       <c r="M286" s="2" t="n">
         <v>0.0</v>
@@ -22867,7 +22867,7 @@
         <v>1401</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>201</v>
+        <v>1401</v>
       </c>
       <c r="D287" s="2" t="n">
         <v>0.0</v>
@@ -22882,25 +22882,25 @@
         <v>0.0</v>
       </c>
       <c r="H287" s="2" t="s">
-        <v>1402</v>
+        <v>1401</v>
       </c>
       <c r="I287" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J287" s="2" t="s">
-        <v>1402</v>
+        <v>1403</v>
       </c>
       <c r="K287" s="2" t="n">
-        <v>1129.0</v>
+        <v>1132.0</v>
       </c>
       <c r="L287" s="2" t="s">
-        <v>1402</v>
+        <v>1404</v>
       </c>
       <c r="M287" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N287" s="2" t="s">
-        <v>1403</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="288">
@@ -22908,16 +22908,16 @@
         <v>287.0</v>
       </c>
       <c r="B288" s="2" t="s">
-        <v>1404</v>
+        <v>1406</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>1405</v>
+        <v>201</v>
       </c>
       <c r="D288" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E288" s="2" t="s">
-        <v>1406</v>
+        <v>1407</v>
       </c>
       <c r="F288" s="2" t="n">
         <v>0.0</v>
@@ -22926,22 +22926,22 @@
         <v>0.0</v>
       </c>
       <c r="H288" s="2" t="s">
-        <v>1406</v>
+        <v>1407</v>
       </c>
       <c r="I288" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J288" s="2" t="s">
-        <v>1406</v>
+        <v>1407</v>
       </c>
       <c r="K288" s="2" t="n">
-        <v>1046.0</v>
+        <v>1129.0</v>
       </c>
       <c r="L288" s="2" t="s">
         <v>1407</v>
       </c>
       <c r="M288" s="2" t="n">
-        <v>8.0</v>
+        <v>0.0</v>
       </c>
       <c r="N288" s="2" t="s">
         <v>1408</v>
@@ -22955,13 +22955,13 @@
         <v>1409</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>201</v>
+        <v>1410</v>
       </c>
       <c r="D289" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E289" s="2" t="s">
-        <v>201</v>
+        <v>1411</v>
       </c>
       <c r="F289" s="2" t="n">
         <v>0.0</v>
@@ -22970,7 +22970,7 @@
         <v>0.0</v>
       </c>
       <c r="H289" s="2" t="s">
-        <v>1410</v>
+        <v>1411</v>
       </c>
       <c r="I289" s="2" t="n">
         <v>0.0</v>
@@ -22979,13 +22979,13 @@
         <v>1411</v>
       </c>
       <c r="K289" s="2" t="n">
-        <v>1102.0</v>
+        <v>1046.0</v>
       </c>
       <c r="L289" s="2" t="s">
         <v>1412</v>
       </c>
       <c r="M289" s="2" t="n">
-        <v>0.0</v>
+        <v>8.0</v>
       </c>
       <c r="N289" s="2" t="s">
         <v>1413</v>
@@ -22999,13 +22999,13 @@
         <v>1414</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>1414</v>
+        <v>201</v>
       </c>
       <c r="D290" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E290" s="2" t="s">
-        <v>1414</v>
+        <v>201</v>
       </c>
       <c r="F290" s="2" t="n">
         <v>0.0</v>
@@ -23023,7 +23023,7 @@
         <v>1416</v>
       </c>
       <c r="K290" s="2" t="n">
-        <v>1095.0</v>
+        <v>1102.0</v>
       </c>
       <c r="L290" s="2" t="s">
         <v>1417</v>
@@ -23043,13 +23043,13 @@
         <v>1419</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>1420</v>
+        <v>1419</v>
       </c>
       <c r="D291" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E291" s="2" t="s">
-        <v>201</v>
+        <v>1419</v>
       </c>
       <c r="F291" s="2" t="n">
         <v>0.0</v>
@@ -23067,16 +23067,16 @@
         <v>1421</v>
       </c>
       <c r="K291" s="2" t="n">
-        <v>1092.0</v>
+        <v>1095.0</v>
       </c>
       <c r="L291" s="2" t="s">
-        <v>1420</v>
+        <v>1422</v>
       </c>
       <c r="M291" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N291" s="2" t="s">
-        <v>1422</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="292">
@@ -23084,16 +23084,16 @@
         <v>291.0</v>
       </c>
       <c r="B292" s="2" t="s">
-        <v>1423</v>
+        <v>1424</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>1424</v>
+        <v>1425</v>
       </c>
       <c r="D292" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E292" s="2" t="s">
-        <v>1424</v>
+        <v>201</v>
       </c>
       <c r="F292" s="2" t="n">
         <v>0.0</v>
@@ -23102,25 +23102,25 @@
         <v>0.0</v>
       </c>
       <c r="H292" s="2" t="s">
-        <v>1424</v>
+        <v>1425</v>
       </c>
       <c r="I292" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J292" s="2" t="s">
-        <v>1424</v>
+        <v>1426</v>
       </c>
       <c r="K292" s="2" t="n">
-        <v>1090.0</v>
+        <v>1092.0</v>
       </c>
       <c r="L292" s="2" t="s">
-        <v>1424</v>
+        <v>1425</v>
       </c>
       <c r="M292" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N292" s="2" t="s">
-        <v>1425</v>
+        <v>1427</v>
       </c>
     </row>
     <row r="293">
@@ -23128,16 +23128,16 @@
         <v>292.0</v>
       </c>
       <c r="B293" s="2" t="s">
-        <v>1426</v>
+        <v>1428</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>1427</v>
+        <v>1429</v>
       </c>
       <c r="D293" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E293" s="2" t="s">
-        <v>1428</v>
+        <v>1429</v>
       </c>
       <c r="F293" s="2" t="n">
         <v>0.0</v>
@@ -23146,7 +23146,7 @@
         <v>0.0</v>
       </c>
       <c r="H293" s="2" t="s">
-        <v>1427</v>
+        <v>1429</v>
       </c>
       <c r="I293" s="2" t="n">
         <v>0.0</v>
@@ -23155,16 +23155,16 @@
         <v>1429</v>
       </c>
       <c r="K293" s="2" t="n">
-        <v>1089.0</v>
+        <v>1090.0</v>
       </c>
       <c r="L293" s="2" t="s">
+        <v>1429</v>
+      </c>
+      <c r="M293" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N293" s="2" t="s">
         <v>1430</v>
-      </c>
-      <c r="M293" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N293" s="2" t="s">
-        <v>1431</v>
       </c>
     </row>
     <row r="294">
@@ -23172,43 +23172,43 @@
         <v>293.0</v>
       </c>
       <c r="B294" s="2" t="s">
+        <v>1431</v>
+      </c>
+      <c r="C294" s="2" t="s">
         <v>1432</v>
       </c>
-      <c r="C294" s="2" t="s">
+      <c r="D294" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E294" s="2" t="s">
         <v>1433</v>
       </c>
-      <c r="D294" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E294" s="2" t="s">
+      <c r="F294" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G294" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H294" s="2" t="s">
+        <v>1432</v>
+      </c>
+      <c r="I294" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J294" s="2" t="s">
         <v>1434</v>
-      </c>
-      <c r="F294" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G294" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H294" s="2" t="s">
-        <v>1435</v>
-      </c>
-      <c r="I294" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J294" s="2" t="s">
-        <v>1436</v>
       </c>
       <c r="K294" s="2" t="n">
         <v>1089.0</v>
       </c>
       <c r="L294" s="2" t="s">
-        <v>1437</v>
+        <v>1435</v>
       </c>
       <c r="M294" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N294" s="2" t="s">
-        <v>1431</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="295">
@@ -23216,43 +23216,43 @@
         <v>294.0</v>
       </c>
       <c r="B295" s="2" t="s">
+        <v>1437</v>
+      </c>
+      <c r="C295" s="2" t="s">
         <v>1438</v>
       </c>
-      <c r="C295" s="2" t="s">
+      <c r="D295" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E295" s="2" t="s">
         <v>1439</v>
       </c>
-      <c r="D295" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E295" s="2" t="s">
+      <c r="F295" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G295" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H295" s="2" t="s">
         <v>1440</v>
       </c>
-      <c r="F295" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G295" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H295" s="2" t="s">
+      <c r="I295" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J295" s="2" t="s">
         <v>1441</v>
       </c>
-      <c r="I295" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J295" s="2" t="s">
+      <c r="K295" s="2" t="n">
+        <v>1089.0</v>
+      </c>
+      <c r="L295" s="2" t="s">
         <v>1442</v>
       </c>
-      <c r="K295" s="2" t="n">
-        <v>1057.0</v>
-      </c>
-      <c r="L295" s="2" t="s">
-        <v>1441</v>
-      </c>
       <c r="M295" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="N295" s="2" t="s">
-        <v>1443</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="296">
@@ -23260,10 +23260,10 @@
         <v>295.0</v>
       </c>
       <c r="B296" s="2" t="s">
+        <v>1443</v>
+      </c>
+      <c r="C296" s="2" t="s">
         <v>1444</v>
-      </c>
-      <c r="C296" s="2" t="s">
-        <v>201</v>
       </c>
       <c r="D296" s="2" t="n">
         <v>0.0</v>
@@ -23284,19 +23284,19 @@
         <v>0.0</v>
       </c>
       <c r="J296" s="2" t="s">
+        <v>1447</v>
+      </c>
+      <c r="K296" s="2" t="n">
+        <v>1057.0</v>
+      </c>
+      <c r="L296" s="2" t="s">
         <v>1446</v>
       </c>
-      <c r="K296" s="2" t="n">
-        <v>1087.0</v>
-      </c>
-      <c r="L296" s="2" t="s">
-        <v>1447</v>
-      </c>
       <c r="M296" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="N296" s="2" t="s">
-        <v>1443</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="297">
@@ -23304,16 +23304,16 @@
         <v>296.0</v>
       </c>
       <c r="B297" s="2" t="s">
-        <v>1448</v>
+        <v>1449</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>1449</v>
+        <v>201</v>
       </c>
       <c r="D297" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E297" s="2" t="s">
-        <v>201</v>
+        <v>1450</v>
       </c>
       <c r="F297" s="2" t="n">
         <v>0.0</v>
@@ -23322,7 +23322,7 @@
         <v>0.0</v>
       </c>
       <c r="H297" s="2" t="s">
-        <v>1450</v>
+        <v>1451</v>
       </c>
       <c r="I297" s="2" t="n">
         <v>0.0</v>
@@ -23331,16 +23331,16 @@
         <v>1451</v>
       </c>
       <c r="K297" s="2" t="n">
-        <v>994.0</v>
+        <v>1087.0</v>
       </c>
       <c r="L297" s="2" t="s">
-        <v>1451</v>
+        <v>1452</v>
       </c>
       <c r="M297" s="2" t="n">
-        <v>12.0</v>
+        <v>0.0</v>
       </c>
       <c r="N297" s="2" t="s">
-        <v>1452</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="298">
@@ -23351,13 +23351,13 @@
         <v>1453</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>201</v>
+        <v>1454</v>
       </c>
       <c r="D298" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E298" s="2" t="s">
-        <v>1454</v>
+        <v>201</v>
       </c>
       <c r="F298" s="2" t="n">
         <v>0.0</v>
@@ -23366,25 +23366,25 @@
         <v>0.0</v>
       </c>
       <c r="H298" s="2" t="s">
-        <v>1454</v>
+        <v>1455</v>
       </c>
       <c r="I298" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J298" s="2" t="s">
-        <v>1455</v>
+        <v>1456</v>
       </c>
       <c r="K298" s="2" t="n">
-        <v>1086.0</v>
+        <v>994.0</v>
       </c>
       <c r="L298" s="2" t="s">
         <v>1456</v>
       </c>
       <c r="M298" s="2" t="n">
-        <v>0.0</v>
+        <v>12.0</v>
       </c>
       <c r="N298" s="2" t="s">
-        <v>1452</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="299">
@@ -23392,43 +23392,43 @@
         <v>298.0</v>
       </c>
       <c r="B299" s="2" t="s">
+        <v>1458</v>
+      </c>
+      <c r="C299" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D299" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E299" s="2" t="s">
+        <v>1459</v>
+      </c>
+      <c r="F299" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G299" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H299" s="2" t="s">
+        <v>1459</v>
+      </c>
+      <c r="I299" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J299" s="2" t="s">
+        <v>1460</v>
+      </c>
+      <c r="K299" s="2" t="n">
+        <v>1086.0</v>
+      </c>
+      <c r="L299" s="2" t="s">
+        <v>1461</v>
+      </c>
+      <c r="M299" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N299" s="2" t="s">
         <v>1457</v>
-      </c>
-      <c r="C299" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="D299" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E299" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F299" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G299" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H299" s="2" t="s">
-        <v>1458</v>
-      </c>
-      <c r="I299" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J299" s="2" t="s">
-        <v>1459</v>
-      </c>
-      <c r="K299" s="2" t="n">
-        <v>802.0</v>
-      </c>
-      <c r="L299" s="2" t="s">
-        <v>1460</v>
-      </c>
-      <c r="M299" s="2" t="n">
-        <v>36.0</v>
-      </c>
-      <c r="N299" s="2" t="s">
-        <v>1461</v>
       </c>
     </row>
     <row r="300">
@@ -23445,16 +23445,16 @@
         <v>0.0</v>
       </c>
       <c r="E300" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F300" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G300" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H300" s="2" t="s">
         <v>1463</v>
-      </c>
-      <c r="F300" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G300" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H300" s="2" t="s">
-        <v>1464</v>
       </c>
       <c r="I300" s="2" t="n">
         <v>0.0</v>
@@ -23463,13 +23463,13 @@
         <v>1464</v>
       </c>
       <c r="K300" s="2" t="n">
-        <v>1076.0</v>
+        <v>802.0</v>
       </c>
       <c r="L300" s="2" t="s">
         <v>1465</v>
       </c>
       <c r="M300" s="2" t="n">
-        <v>0.0</v>
+        <v>36.0</v>
       </c>
       <c r="N300" s="2" t="s">
         <v>1466</v>
@@ -23483,40 +23483,40 @@
         <v>1467</v>
       </c>
       <c r="C301" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D301" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E301" s="2" t="s">
         <v>1468</v>
       </c>
-      <c r="D301" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E301" s="2" t="s">
+      <c r="F301" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G301" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H301" s="2" t="s">
         <v>1469</v>
       </c>
-      <c r="F301" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G301" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H301" s="2" t="s">
+      <c r="I301" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J301" s="2" t="s">
+        <v>1469</v>
+      </c>
+      <c r="K301" s="2" t="n">
+        <v>1076.0</v>
+      </c>
+      <c r="L301" s="2" t="s">
         <v>1470</v>
       </c>
-      <c r="I301" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J301" s="2" t="s">
+      <c r="M301" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N301" s="2" t="s">
         <v>1471</v>
-      </c>
-      <c r="K301" s="2" t="n">
-        <v>1034.0</v>
-      </c>
-      <c r="L301" s="2" t="s">
-        <v>1468</v>
-      </c>
-      <c r="M301" s="2" t="n">
-        <v>5.0</v>
-      </c>
-      <c r="N301" s="2" t="s">
-        <v>1472</v>
       </c>
     </row>
     <row r="302">
@@ -23524,43 +23524,43 @@
         <v>301.0</v>
       </c>
       <c r="B302" s="2" t="s">
+        <v>1472</v>
+      </c>
+      <c r="C302" s="2" t="s">
         <v>1473</v>
       </c>
-      <c r="C302" s="2" t="s">
+      <c r="D302" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E302" s="2" t="s">
         <v>1474</v>
       </c>
-      <c r="D302" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E302" s="2" t="s">
+      <c r="F302" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G302" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H302" s="2" t="s">
         <v>1475</v>
       </c>
-      <c r="F302" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G302" s="2" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="H302" s="2" t="s">
+      <c r="I302" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J302" s="2" t="s">
         <v>1476</v>
       </c>
-      <c r="I302" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J302" s="2" t="s">
+      <c r="K302" s="2" t="n">
+        <v>1034.0</v>
+      </c>
+      <c r="L302" s="2" t="s">
+        <v>1473</v>
+      </c>
+      <c r="M302" s="2" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="N302" s="2" t="s">
         <v>1477</v>
-      </c>
-      <c r="K302" s="2" t="n">
-        <v>1060.0</v>
-      </c>
-      <c r="L302" s="2" t="s">
-        <v>1474</v>
-      </c>
-      <c r="M302" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N302" s="2" t="s">
-        <v>1478</v>
       </c>
     </row>
     <row r="303">
@@ -23568,25 +23568,25 @@
         <v>302.0</v>
       </c>
       <c r="B303" s="2" t="s">
+        <v>1478</v>
+      </c>
+      <c r="C303" s="2" t="s">
         <v>1479</v>
       </c>
-      <c r="C303" s="2" t="s">
+      <c r="D303" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E303" s="2" t="s">
         <v>1480</v>
       </c>
-      <c r="D303" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E303" s="2" t="s">
+      <c r="F303" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G303" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="H303" s="2" t="s">
         <v>1481</v>
-      </c>
-      <c r="F303" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G303" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H303" s="2" t="s">
-        <v>1480</v>
       </c>
       <c r="I303" s="2" t="n">
         <v>0.0</v>
@@ -23595,10 +23595,10 @@
         <v>1482</v>
       </c>
       <c r="K303" s="2" t="n">
-        <v>1058.0</v>
+        <v>1060.0</v>
       </c>
       <c r="L303" s="2" t="s">
-        <v>1480</v>
+        <v>1479</v>
       </c>
       <c r="M303" s="2" t="n">
         <v>0.0</v>
@@ -23621,13 +23621,13 @@
         <v>0.0</v>
       </c>
       <c r="E304" s="2" t="s">
-        <v>1485</v>
+        <v>1486</v>
       </c>
       <c r="F304" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G304" s="2" t="n">
-        <v>5.0</v>
+        <v>0.0</v>
       </c>
       <c r="H304" s="2" t="s">
         <v>1485</v>
@@ -23636,19 +23636,19 @@
         <v>0.0</v>
       </c>
       <c r="J304" s="2" t="s">
-        <v>1486</v>
+        <v>1487</v>
       </c>
       <c r="K304" s="2" t="n">
-        <v>986.0</v>
+        <v>1058.0</v>
       </c>
       <c r="L304" s="2" t="s">
         <v>1485</v>
       </c>
       <c r="M304" s="2" t="n">
-        <v>8.0</v>
+        <v>0.0</v>
       </c>
       <c r="N304" s="2" t="s">
-        <v>1487</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="305">
@@ -23656,22 +23656,22 @@
         <v>304.0</v>
       </c>
       <c r="B305" s="2" t="s">
-        <v>1488</v>
+        <v>1489</v>
       </c>
       <c r="C305" s="2" t="s">
-        <v>1489</v>
+        <v>1490</v>
       </c>
       <c r="D305" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E305" s="2" t="s">
-        <v>1489</v>
+        <v>1490</v>
       </c>
       <c r="F305" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G305" s="2" t="n">
-        <v>0.0</v>
+        <v>5.0</v>
       </c>
       <c r="H305" s="2" t="s">
         <v>1490</v>
@@ -23680,19 +23680,19 @@
         <v>0.0</v>
       </c>
       <c r="J305" s="2" t="s">
+        <v>1491</v>
+      </c>
+      <c r="K305" s="2" t="n">
+        <v>986.0</v>
+      </c>
+      <c r="L305" s="2" t="s">
         <v>1490</v>
       </c>
-      <c r="K305" s="2" t="n">
-        <v>948.0</v>
-      </c>
-      <c r="L305" s="2" t="s">
-        <v>1489</v>
-      </c>
       <c r="M305" s="2" t="n">
-        <v>13.0</v>
+        <v>8.0</v>
       </c>
       <c r="N305" s="2" t="s">
-        <v>1491</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="306">
@@ -23700,10 +23700,10 @@
         <v>305.0</v>
       </c>
       <c r="B306" s="2" t="s">
-        <v>1492</v>
+        <v>1493</v>
       </c>
       <c r="C306" s="2" t="s">
-        <v>1493</v>
+        <v>1494</v>
       </c>
       <c r="D306" s="2" t="n">
         <v>0.0</v>
@@ -23724,19 +23724,19 @@
         <v>0.0</v>
       </c>
       <c r="J306" s="2" t="s">
-        <v>1493</v>
+        <v>1495</v>
       </c>
       <c r="K306" s="2" t="n">
-        <v>1048.0</v>
+        <v>948.0</v>
       </c>
       <c r="L306" s="2" t="s">
-        <v>1495</v>
+        <v>1494</v>
       </c>
       <c r="M306" s="2" t="n">
-        <v>0.0</v>
+        <v>13.0</v>
       </c>
       <c r="N306" s="2" t="s">
-        <v>1491</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="307">
@@ -23744,43 +23744,43 @@
         <v>306.0</v>
       </c>
       <c r="B307" s="2" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C307" s="2" t="s">
+        <v>1498</v>
+      </c>
+      <c r="D307" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E307" s="2" t="s">
+        <v>1499</v>
+      </c>
+      <c r="F307" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G307" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H307" s="2" t="s">
+        <v>1500</v>
+      </c>
+      <c r="I307" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J307" s="2" t="s">
+        <v>1498</v>
+      </c>
+      <c r="K307" s="2" t="n">
+        <v>1048.0</v>
+      </c>
+      <c r="L307" s="2" t="s">
+        <v>1500</v>
+      </c>
+      <c r="M307" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N307" s="2" t="s">
         <v>1496</v>
-      </c>
-      <c r="C307" s="2" t="s">
-        <v>1497</v>
-      </c>
-      <c r="D307" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E307" s="2" t="s">
-        <v>1498</v>
-      </c>
-      <c r="F307" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G307" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H307" s="2" t="s">
-        <v>1496</v>
-      </c>
-      <c r="I307" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J307" s="2" t="s">
-        <v>1499</v>
-      </c>
-      <c r="K307" s="2" t="n">
-        <v>1047.0</v>
-      </c>
-      <c r="L307" s="2" t="s">
-        <v>1497</v>
-      </c>
-      <c r="M307" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N307" s="2" t="s">
-        <v>1491</v>
       </c>
     </row>
     <row r="308">
@@ -23788,43 +23788,43 @@
         <v>307.0</v>
       </c>
       <c r="B308" s="2" t="s">
-        <v>1500</v>
+        <v>1501</v>
       </c>
       <c r="C308" s="2" t="s">
-        <v>201</v>
+        <v>1502</v>
       </c>
       <c r="D308" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E308" s="2" t="s">
+        <v>1503</v>
+      </c>
+      <c r="F308" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G308" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H308" s="2" t="s">
         <v>1501</v>
       </c>
-      <c r="F308" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G308" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H308" s="2" t="s">
+      <c r="I308" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J308" s="2" t="s">
+        <v>1504</v>
+      </c>
+      <c r="K308" s="2" t="n">
+        <v>1047.0</v>
+      </c>
+      <c r="L308" s="2" t="s">
         <v>1502</v>
       </c>
-      <c r="I308" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J308" s="2" t="s">
-        <v>1503</v>
-      </c>
-      <c r="K308" s="2" t="n">
-        <v>1042.0</v>
-      </c>
-      <c r="L308" s="2" t="s">
-        <v>201</v>
-      </c>
       <c r="M308" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N308" s="2" t="s">
-        <v>1504</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="309">
@@ -23835,13 +23835,13 @@
         <v>1505</v>
       </c>
       <c r="C309" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D309" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E309" s="2" t="s">
         <v>1506</v>
-      </c>
-      <c r="D309" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E309" s="2" t="s">
-        <v>201</v>
       </c>
       <c r="F309" s="2" t="n">
         <v>0.0</v>
@@ -23859,16 +23859,16 @@
         <v>1508</v>
       </c>
       <c r="K309" s="2" t="n">
-        <v>1041.0</v>
+        <v>1042.0</v>
       </c>
       <c r="L309" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="M309" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N309" s="2" t="s">
         <v>1509</v>
-      </c>
-      <c r="M309" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N309" s="2" t="s">
-        <v>1510</v>
       </c>
     </row>
     <row r="310">
@@ -23876,10 +23876,10 @@
         <v>309.0</v>
       </c>
       <c r="B310" s="2" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C310" s="2" t="s">
         <v>1511</v>
-      </c>
-      <c r="C310" s="2" t="s">
-        <v>1512</v>
       </c>
       <c r="D310" s="2" t="n">
         <v>0.0</v>
@@ -23903,16 +23903,16 @@
         <v>1513</v>
       </c>
       <c r="K310" s="2" t="n">
-        <v>1034.0</v>
+        <v>1041.0</v>
       </c>
       <c r="L310" s="2" t="s">
-        <v>1513</v>
+        <v>1514</v>
       </c>
       <c r="M310" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N310" s="2" t="s">
-        <v>1514</v>
+        <v>1515</v>
       </c>
     </row>
     <row r="311">
@@ -23920,16 +23920,16 @@
         <v>310.0</v>
       </c>
       <c r="B311" s="2" t="s">
-        <v>1515</v>
+        <v>1516</v>
       </c>
       <c r="C311" s="2" t="s">
-        <v>201</v>
+        <v>1517</v>
       </c>
       <c r="D311" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E311" s="2" t="s">
-        <v>1516</v>
+        <v>201</v>
       </c>
       <c r="F311" s="2" t="n">
         <v>0.0</v>
@@ -23938,25 +23938,25 @@
         <v>0.0</v>
       </c>
       <c r="H311" s="2" t="s">
-        <v>201</v>
+        <v>1517</v>
       </c>
       <c r="I311" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J311" s="2" t="s">
-        <v>1517</v>
+        <v>1518</v>
       </c>
       <c r="K311" s="2" t="n">
-        <v>1031.0</v>
+        <v>1034.0</v>
       </c>
       <c r="L311" s="2" t="s">
-        <v>201</v>
+        <v>1518</v>
       </c>
       <c r="M311" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N311" s="2" t="s">
-        <v>1518</v>
+        <v>1519</v>
       </c>
     </row>
     <row r="312">
@@ -23964,16 +23964,16 @@
         <v>311.0</v>
       </c>
       <c r="B312" s="2" t="s">
-        <v>1519</v>
+        <v>1520</v>
       </c>
       <c r="C312" s="2" t="s">
-        <v>1520</v>
+        <v>201</v>
       </c>
       <c r="D312" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E312" s="2" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="F312" s="2" t="n">
         <v>0.0</v>
@@ -23982,25 +23982,25 @@
         <v>0.0</v>
       </c>
       <c r="H312" s="2" t="s">
-        <v>1520</v>
+        <v>201</v>
       </c>
       <c r="I312" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J312" s="2" t="s">
-        <v>1521</v>
+        <v>1522</v>
       </c>
       <c r="K312" s="2" t="n">
-        <v>933.0</v>
+        <v>1031.0</v>
       </c>
       <c r="L312" s="2" t="s">
-        <v>1520</v>
+        <v>201</v>
       </c>
       <c r="M312" s="2" t="n">
-        <v>12.0</v>
+        <v>0.0</v>
       </c>
       <c r="N312" s="2" t="s">
-        <v>1522</v>
+        <v>1523</v>
       </c>
     </row>
     <row r="313">
@@ -24008,16 +24008,16 @@
         <v>312.0</v>
       </c>
       <c r="B313" s="2" t="s">
-        <v>1523</v>
+        <v>1524</v>
       </c>
       <c r="C313" s="2" t="s">
-        <v>1524</v>
+        <v>1525</v>
       </c>
       <c r="D313" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E313" s="2" t="s">
-        <v>201</v>
+        <v>1525</v>
       </c>
       <c r="F313" s="2" t="n">
         <v>0.0</v>
@@ -24032,16 +24032,16 @@
         <v>0.0</v>
       </c>
       <c r="J313" s="2" t="s">
+        <v>1526</v>
+      </c>
+      <c r="K313" s="2" t="n">
+        <v>933.0</v>
+      </c>
+      <c r="L313" s="2" t="s">
         <v>1525</v>
       </c>
-      <c r="K313" s="2" t="n">
-        <v>1020.0</v>
-      </c>
-      <c r="L313" s="2" t="s">
-        <v>1526</v>
-      </c>
       <c r="M313" s="2" t="n">
-        <v>0.0</v>
+        <v>12.0</v>
       </c>
       <c r="N313" s="2" t="s">
         <v>1527</v>
@@ -24061,34 +24061,34 @@
         <v>0.0</v>
       </c>
       <c r="E314" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F314" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G314" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H314" s="2" t="s">
         <v>1530</v>
       </c>
-      <c r="F314" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G314" s="2" t="n">
-        <v>85.0</v>
-      </c>
-      <c r="H314" s="2" t="s">
+      <c r="I314" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J314" s="2" t="s">
+        <v>1530</v>
+      </c>
+      <c r="K314" s="2" t="n">
+        <v>1020.0</v>
+      </c>
+      <c r="L314" s="2" t="s">
         <v>1531</v>
       </c>
-      <c r="I314" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J314" s="2" t="s">
-        <v>1529</v>
-      </c>
-      <c r="K314" s="2" t="n">
-        <v>889.0</v>
-      </c>
-      <c r="L314" s="2" t="s">
+      <c r="M314" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N314" s="2" t="s">
         <v>1532</v>
-      </c>
-      <c r="M314" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N314" s="2" t="s">
-        <v>1533</v>
       </c>
     </row>
     <row r="315">
@@ -24096,34 +24096,34 @@
         <v>314.0</v>
       </c>
       <c r="B315" s="2" t="s">
+        <v>1533</v>
+      </c>
+      <c r="C315" s="2" t="s">
         <v>1534</v>
       </c>
-      <c r="C315" s="2" t="s">
-        <v>201</v>
-      </c>
       <c r="D315" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E315" s="2" t="s">
-        <v>201</v>
+        <v>1535</v>
       </c>
       <c r="F315" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G315" s="2" t="n">
-        <v>0.0</v>
+        <v>85.0</v>
       </c>
       <c r="H315" s="2" t="s">
-        <v>1535</v>
+        <v>1536</v>
       </c>
       <c r="I315" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J315" s="2" t="s">
-        <v>1536</v>
+        <v>1534</v>
       </c>
       <c r="K315" s="2" t="n">
-        <v>1018.0</v>
+        <v>889.0</v>
       </c>
       <c r="L315" s="2" t="s">
         <v>1537</v>
@@ -24132,7 +24132,7 @@
         <v>0.0</v>
       </c>
       <c r="N315" s="2" t="s">
-        <v>1533</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="316">
@@ -24140,43 +24140,43 @@
         <v>315.0</v>
       </c>
       <c r="B316" s="2" t="s">
+        <v>1539</v>
+      </c>
+      <c r="C316" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D316" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E316" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F316" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G316" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H316" s="2" t="s">
+        <v>1540</v>
+      </c>
+      <c r="I316" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J316" s="2" t="s">
+        <v>1541</v>
+      </c>
+      <c r="K316" s="2" t="n">
+        <v>1018.0</v>
+      </c>
+      <c r="L316" s="2" t="s">
+        <v>1542</v>
+      </c>
+      <c r="M316" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N316" s="2" t="s">
         <v>1538</v>
-      </c>
-      <c r="C316" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="D316" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E316" s="2" t="s">
-        <v>1539</v>
-      </c>
-      <c r="F316" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G316" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H316" s="2" t="s">
-        <v>1538</v>
-      </c>
-      <c r="I316" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J316" s="2" t="s">
-        <v>1540</v>
-      </c>
-      <c r="K316" s="2" t="n">
-        <v>1017.0</v>
-      </c>
-      <c r="L316" s="2" t="s">
-        <v>1539</v>
-      </c>
-      <c r="M316" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N316" s="2" t="s">
-        <v>1541</v>
       </c>
     </row>
     <row r="317">
@@ -24184,10 +24184,10 @@
         <v>316.0</v>
       </c>
       <c r="B317" s="2" t="s">
-        <v>1542</v>
+        <v>1543</v>
       </c>
       <c r="C317" s="2" t="s">
-        <v>1543</v>
+        <v>201</v>
       </c>
       <c r="D317" s="2" t="n">
         <v>0.0</v>
@@ -24202,25 +24202,25 @@
         <v>0.0</v>
       </c>
       <c r="H317" s="2" t="s">
+        <v>1543</v>
+      </c>
+      <c r="I317" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J317" s="2" t="s">
         <v>1545</v>
       </c>
-      <c r="I317" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J317" s="2" t="s">
+      <c r="K317" s="2" t="n">
+        <v>1017.0</v>
+      </c>
+      <c r="L317" s="2" t="s">
+        <v>1544</v>
+      </c>
+      <c r="M317" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N317" s="2" t="s">
         <v>1546</v>
-      </c>
-      <c r="K317" s="2" t="n">
-        <v>1015.0</v>
-      </c>
-      <c r="L317" s="2" t="s">
-        <v>1547</v>
-      </c>
-      <c r="M317" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N317" s="2" t="s">
-        <v>1548</v>
       </c>
     </row>
     <row r="318">
@@ -24228,37 +24228,37 @@
         <v>317.0</v>
       </c>
       <c r="B318" s="2" t="s">
+        <v>1547</v>
+      </c>
+      <c r="C318" s="2" t="s">
+        <v>1548</v>
+      </c>
+      <c r="D318" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E318" s="2" t="s">
         <v>1549</v>
       </c>
-      <c r="C318" s="2" t="s">
+      <c r="F318" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G318" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H318" s="2" t="s">
         <v>1550</v>
       </c>
-      <c r="D318" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E318" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="F318" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G318" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H318" s="2" t="s">
+      <c r="I318" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J318" s="2" t="s">
         <v>1551</v>
       </c>
-      <c r="I318" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J318" s="2" t="s">
+      <c r="K318" s="2" t="n">
+        <v>1015.0</v>
+      </c>
+      <c r="L318" s="2" t="s">
         <v>1552</v>
-      </c>
-      <c r="K318" s="2" t="n">
-        <v>1009.0</v>
-      </c>
-      <c r="L318" s="2" t="s">
-        <v>1549</v>
       </c>
       <c r="M318" s="2" t="n">
         <v>0.0</v>
@@ -24275,13 +24275,13 @@
         <v>1554</v>
       </c>
       <c r="C319" s="2" t="s">
-        <v>1554</v>
+        <v>1555</v>
       </c>
       <c r="D319" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E319" s="2" t="s">
-        <v>1555</v>
+        <v>201</v>
       </c>
       <c r="F319" s="2" t="n">
         <v>0.0</v>
@@ -24290,16 +24290,16 @@
         <v>0.0</v>
       </c>
       <c r="H319" s="2" t="s">
-        <v>1554</v>
+        <v>1556</v>
       </c>
       <c r="I319" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J319" s="2" t="s">
-        <v>1556</v>
+        <v>1557</v>
       </c>
       <c r="K319" s="2" t="n">
-        <v>1008.0</v>
+        <v>1009.0</v>
       </c>
       <c r="L319" s="2" t="s">
         <v>1554</v>
@@ -24308,7 +24308,7 @@
         <v>0.0</v>
       </c>
       <c r="N319" s="2" t="s">
-        <v>1553</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="320">
@@ -24316,43 +24316,43 @@
         <v>319.0</v>
       </c>
       <c r="B320" s="2" t="s">
-        <v>1557</v>
+        <v>1559</v>
       </c>
       <c r="C320" s="2" t="s">
-        <v>201</v>
+        <v>1559</v>
       </c>
       <c r="D320" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E320" s="2" t="s">
+        <v>1560</v>
+      </c>
+      <c r="F320" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G320" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H320" s="2" t="s">
+        <v>1559</v>
+      </c>
+      <c r="I320" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J320" s="2" t="s">
+        <v>1561</v>
+      </c>
+      <c r="K320" s="2" t="n">
+        <v>1008.0</v>
+      </c>
+      <c r="L320" s="2" t="s">
+        <v>1559</v>
+      </c>
+      <c r="M320" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N320" s="2" t="s">
         <v>1558</v>
-      </c>
-      <c r="F320" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G320" s="2" t="n">
-        <v>7.0</v>
-      </c>
-      <c r="H320" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="I320" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J320" s="2" t="s">
-        <v>1559</v>
-      </c>
-      <c r="K320" s="2" t="n">
-        <v>997.0</v>
-      </c>
-      <c r="L320" s="2" t="s">
-        <v>1558</v>
-      </c>
-      <c r="M320" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N320" s="2" t="s">
-        <v>1560</v>
       </c>
     </row>
     <row r="321">
@@ -24360,7 +24360,7 @@
         <v>320.0</v>
       </c>
       <c r="B321" s="2" t="s">
-        <v>1561</v>
+        <v>1562</v>
       </c>
       <c r="C321" s="2" t="s">
         <v>201</v>
@@ -24369,25 +24369,25 @@
         <v>0.0</v>
       </c>
       <c r="E321" s="2" t="s">
-        <v>1562</v>
+        <v>1563</v>
       </c>
       <c r="F321" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G321" s="2" t="n">
-        <v>0.0</v>
+        <v>7.0</v>
       </c>
       <c r="H321" s="2" t="s">
-        <v>1562</v>
+        <v>201</v>
       </c>
       <c r="I321" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J321" s="2" t="s">
-        <v>1562</v>
+        <v>1564</v>
       </c>
       <c r="K321" s="2" t="n">
-        <v>1006.0</v>
+        <v>997.0</v>
       </c>
       <c r="L321" s="2" t="s">
         <v>1563</v>
@@ -24396,7 +24396,7 @@
         <v>0.0</v>
       </c>
       <c r="N321" s="2" t="s">
-        <v>1564</v>
+        <v>1565</v>
       </c>
     </row>
     <row r="322">
@@ -24404,10 +24404,10 @@
         <v>321.0</v>
       </c>
       <c r="B322" s="2" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
       <c r="C322" s="2" t="s">
-        <v>1566</v>
+        <v>201</v>
       </c>
       <c r="D322" s="2" t="n">
         <v>0.0</v>
@@ -24422,25 +24422,25 @@
         <v>0.0</v>
       </c>
       <c r="H322" s="2" t="s">
+        <v>1567</v>
+      </c>
+      <c r="I322" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J322" s="2" t="s">
+        <v>1567</v>
+      </c>
+      <c r="K322" s="2" t="n">
+        <v>1006.0</v>
+      </c>
+      <c r="L322" s="2" t="s">
         <v>1568</v>
       </c>
-      <c r="I322" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J322" s="2" t="s">
+      <c r="M322" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N322" s="2" t="s">
         <v>1569</v>
-      </c>
-      <c r="K322" s="2" t="n">
-        <v>1004.0</v>
-      </c>
-      <c r="L322" s="2" t="s">
-        <v>1566</v>
-      </c>
-      <c r="M322" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N322" s="2" t="s">
-        <v>1570</v>
       </c>
     </row>
     <row r="323">
@@ -24448,43 +24448,43 @@
         <v>322.0</v>
       </c>
       <c r="B323" s="2" t="s">
+        <v>1570</v>
+      </c>
+      <c r="C323" s="2" t="s">
         <v>1571</v>
       </c>
-      <c r="C323" s="2" t="s">
+      <c r="D323" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E323" s="2" t="s">
         <v>1572</v>
       </c>
-      <c r="D323" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E323" s="2" t="s">
+      <c r="F323" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G323" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H323" s="2" t="s">
         <v>1573</v>
       </c>
-      <c r="F323" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G323" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H323" s="2" t="s">
+      <c r="I323" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J323" s="2" t="s">
         <v>1574</v>
       </c>
-      <c r="I323" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J323" s="2" t="s">
+      <c r="K323" s="2" t="n">
+        <v>1004.0</v>
+      </c>
+      <c r="L323" s="2" t="s">
+        <v>1571</v>
+      </c>
+      <c r="M323" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N323" s="2" t="s">
         <v>1575</v>
-      </c>
-      <c r="K323" s="2" t="n">
-        <v>1003.0</v>
-      </c>
-      <c r="L323" s="2" t="s">
-        <v>1572</v>
-      </c>
-      <c r="M323" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N323" s="2" t="s">
-        <v>1576</v>
       </c>
     </row>
     <row r="324">
@@ -24492,10 +24492,10 @@
         <v>323.0</v>
       </c>
       <c r="B324" s="2" t="s">
+        <v>1576</v>
+      </c>
+      <c r="C324" s="2" t="s">
         <v>1577</v>
-      </c>
-      <c r="C324" s="2" t="s">
-        <v>201</v>
       </c>
       <c r="D324" s="2" t="n">
         <v>0.0</v>
@@ -24510,25 +24510,25 @@
         <v>0.0</v>
       </c>
       <c r="H324" s="2" t="s">
-        <v>201</v>
+        <v>1579</v>
       </c>
       <c r="I324" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J324" s="2" t="s">
-        <v>1579</v>
+        <v>1580</v>
       </c>
       <c r="K324" s="2" t="n">
-        <v>1001.0</v>
+        <v>1003.0</v>
       </c>
       <c r="L324" s="2" t="s">
-        <v>1578</v>
+        <v>1577</v>
       </c>
       <c r="M324" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N324" s="2" t="s">
-        <v>1580</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="325">
@@ -24536,10 +24536,10 @@
         <v>324.0</v>
       </c>
       <c r="B325" s="2" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="C325" s="2" t="s">
-        <v>1582</v>
+        <v>201</v>
       </c>
       <c r="D325" s="2" t="n">
         <v>0.0</v>
@@ -24554,25 +24554,25 @@
         <v>0.0</v>
       </c>
       <c r="H325" s="2" t="s">
-        <v>1582</v>
+        <v>201</v>
       </c>
       <c r="I325" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J325" s="2" t="s">
-        <v>1582</v>
+        <v>1584</v>
       </c>
       <c r="K325" s="2" t="n">
         <v>1001.0</v>
       </c>
       <c r="L325" s="2" t="s">
-        <v>1584</v>
+        <v>1583</v>
       </c>
       <c r="M325" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N325" s="2" t="s">
-        <v>1580</v>
+        <v>1585</v>
       </c>
     </row>
     <row r="326">
@@ -24580,43 +24580,43 @@
         <v>325.0</v>
       </c>
       <c r="B326" s="2" t="s">
+        <v>1586</v>
+      </c>
+      <c r="C326" s="2" t="s">
+        <v>1587</v>
+      </c>
+      <c r="D326" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E326" s="2" t="s">
+        <v>1588</v>
+      </c>
+      <c r="F326" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G326" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H326" s="2" t="s">
+        <v>1587</v>
+      </c>
+      <c r="I326" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J326" s="2" t="s">
+        <v>1587</v>
+      </c>
+      <c r="K326" s="2" t="n">
+        <v>1001.0</v>
+      </c>
+      <c r="L326" s="2" t="s">
+        <v>1589</v>
+      </c>
+      <c r="M326" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N326" s="2" t="s">
         <v>1585</v>
-      </c>
-      <c r="C326" s="2" t="s">
-        <v>1586</v>
-      </c>
-      <c r="D326" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E326" s="2" t="s">
-        <v>1586</v>
-      </c>
-      <c r="F326" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G326" s="2" t="n">
-        <v>12.0</v>
-      </c>
-      <c r="H326" s="2" t="s">
-        <v>1586</v>
-      </c>
-      <c r="I326" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J326" s="2" t="s">
-        <v>1586</v>
-      </c>
-      <c r="K326" s="2" t="n">
-        <v>982.0</v>
-      </c>
-      <c r="L326" s="2" t="s">
-        <v>1587</v>
-      </c>
-      <c r="M326" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N326" s="2" t="s">
-        <v>1580</v>
       </c>
     </row>
     <row r="327">
@@ -24624,43 +24624,43 @@
         <v>326.0</v>
       </c>
       <c r="B327" s="2" t="s">
-        <v>1588</v>
+        <v>1590</v>
       </c>
       <c r="C327" s="2" t="s">
-        <v>201</v>
+        <v>1591</v>
       </c>
       <c r="D327" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E327" s="2" t="s">
-        <v>201</v>
+        <v>1591</v>
       </c>
       <c r="F327" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G327" s="2" t="n">
-        <v>0.0</v>
+        <v>12.0</v>
       </c>
       <c r="H327" s="2" t="s">
-        <v>1589</v>
+        <v>1591</v>
       </c>
       <c r="I327" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J327" s="2" t="s">
-        <v>1590</v>
+        <v>1591</v>
       </c>
       <c r="K327" s="2" t="n">
-        <v>1000.0</v>
+        <v>982.0</v>
       </c>
       <c r="L327" s="2" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="M327" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N327" s="2" t="s">
-        <v>1592</v>
+        <v>1585</v>
       </c>
     </row>
     <row r="328">
@@ -24671,13 +24671,13 @@
         <v>1593</v>
       </c>
       <c r="C328" s="2" t="s">
-        <v>1594</v>
+        <v>201</v>
       </c>
       <c r="D328" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E328" s="2" t="s">
-        <v>1594</v>
+        <v>201</v>
       </c>
       <c r="F328" s="2" t="n">
         <v>0.0</v>
@@ -24692,19 +24692,19 @@
         <v>0.0</v>
       </c>
       <c r="J328" s="2" t="s">
-        <v>1594</v>
+        <v>1595</v>
       </c>
       <c r="K328" s="2" t="n">
-        <v>998.0</v>
+        <v>1000.0</v>
       </c>
       <c r="L328" s="2" t="s">
-        <v>1594</v>
+        <v>1596</v>
       </c>
       <c r="M328" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N328" s="2" t="s">
-        <v>1595</v>
+        <v>1597</v>
       </c>
     </row>
     <row r="329">
@@ -24712,16 +24712,16 @@
         <v>328.0</v>
       </c>
       <c r="B329" s="2" t="s">
-        <v>1596</v>
+        <v>1598</v>
       </c>
       <c r="C329" s="2" t="s">
-        <v>1597</v>
+        <v>1599</v>
       </c>
       <c r="D329" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E329" s="2" t="s">
-        <v>1597</v>
+        <v>1599</v>
       </c>
       <c r="F329" s="2" t="n">
         <v>0.0</v>
@@ -24730,16 +24730,16 @@
         <v>0.0</v>
       </c>
       <c r="H329" s="2" t="s">
-        <v>1597</v>
+        <v>1599</v>
       </c>
       <c r="I329" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J329" s="2" t="s">
-        <v>1598</v>
+        <v>1599</v>
       </c>
       <c r="K329" s="2" t="n">
-        <v>997.0</v>
+        <v>998.0</v>
       </c>
       <c r="L329" s="2" t="s">
         <v>1599</v>
@@ -24765,34 +24765,34 @@
         <v>0.0</v>
       </c>
       <c r="E330" s="2" t="s">
+        <v>1602</v>
+      </c>
+      <c r="F330" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G330" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H330" s="2" t="s">
+        <v>1602</v>
+      </c>
+      <c r="I330" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J330" s="2" t="s">
         <v>1603</v>
       </c>
-      <c r="F330" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G330" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H330" s="2" t="s">
+      <c r="K330" s="2" t="n">
+        <v>997.0</v>
+      </c>
+      <c r="L330" s="2" t="s">
         <v>1604</v>
       </c>
-      <c r="I330" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J330" s="2" t="s">
+      <c r="M330" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N330" s="2" t="s">
         <v>1605</v>
-      </c>
-      <c r="K330" s="2" t="n">
-        <v>902.0</v>
-      </c>
-      <c r="L330" s="2" t="s">
-        <v>1602</v>
-      </c>
-      <c r="M330" s="2" t="n">
-        <v>12.0</v>
-      </c>
-      <c r="N330" s="2" t="s">
-        <v>1606</v>
       </c>
     </row>
     <row r="331">
@@ -24800,17 +24800,17 @@
         <v>330.0</v>
       </c>
       <c r="B331" s="2" t="s">
+        <v>1606</v>
+      </c>
+      <c r="C331" s="2" t="s">
         <v>1607</v>
       </c>
-      <c r="C331" s="2" t="s">
+      <c r="D331" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E331" s="2" t="s">
         <v>1608</v>
       </c>
-      <c r="D331" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E331" s="2" t="s">
-        <v>201</v>
-      </c>
       <c r="F331" s="2" t="n">
         <v>0.0</v>
       </c>
@@ -24818,25 +24818,25 @@
         <v>0.0</v>
       </c>
       <c r="H331" s="2" t="s">
-        <v>201</v>
+        <v>1609</v>
       </c>
       <c r="I331" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J331" s="2" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
       <c r="K331" s="2" t="n">
-        <v>993.0</v>
+        <v>902.0</v>
       </c>
       <c r="L331" s="2" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="M331" s="2" t="n">
-        <v>0.0</v>
+        <v>12.0</v>
       </c>
       <c r="N331" s="2" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="332">
@@ -24844,10 +24844,10 @@
         <v>331.0</v>
       </c>
       <c r="B332" s="2" t="s">
-        <v>1611</v>
+        <v>1612</v>
       </c>
       <c r="C332" s="2" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="D332" s="2" t="n">
         <v>0.0</v>
@@ -24862,7 +24862,7 @@
         <v>0.0</v>
       </c>
       <c r="H332" s="2" t="s">
-        <v>1613</v>
+        <v>201</v>
       </c>
       <c r="I332" s="2" t="n">
         <v>0.0</v>
@@ -24871,10 +24871,10 @@
         <v>1614</v>
       </c>
       <c r="K332" s="2" t="n">
-        <v>991.0</v>
+        <v>993.0</v>
       </c>
       <c r="L332" s="2" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="M332" s="2" t="n">
         <v>0.0</v>
@@ -24897,28 +24897,28 @@
         <v>0.0</v>
       </c>
       <c r="E333" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F333" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G333" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H333" s="2" t="s">
         <v>1618</v>
       </c>
-      <c r="F333" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G333" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H333" s="2" t="s">
+      <c r="I333" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J333" s="2" t="s">
         <v>1619</v>
       </c>
-      <c r="I333" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J333" s="2" t="s">
+      <c r="K333" s="2" t="n">
+        <v>991.0</v>
+      </c>
+      <c r="L333" s="2" t="s">
         <v>1617</v>
-      </c>
-      <c r="K333" s="2" t="n">
-        <v>990.0</v>
-      </c>
-      <c r="L333" s="2" t="s">
-        <v>1619</v>
       </c>
       <c r="M333" s="2" t="n">
         <v>0.0</v>
@@ -24950,7 +24950,7 @@
         <v>0.0</v>
       </c>
       <c r="H334" s="2" t="s">
-        <v>1622</v>
+        <v>1624</v>
       </c>
       <c r="I334" s="2" t="n">
         <v>0.0</v>
@@ -24968,7 +24968,7 @@
         <v>0.0</v>
       </c>
       <c r="N334" s="2" t="s">
-        <v>1620</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="335">
@@ -24976,43 +24976,43 @@
         <v>334.0</v>
       </c>
       <c r="B335" s="2" t="s">
+        <v>1626</v>
+      </c>
+      <c r="C335" s="2" t="s">
+        <v>1627</v>
+      </c>
+      <c r="D335" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E335" s="2" t="s">
+        <v>1628</v>
+      </c>
+      <c r="F335" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G335" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H335" s="2" t="s">
+        <v>1627</v>
+      </c>
+      <c r="I335" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J335" s="2" t="s">
+        <v>1627</v>
+      </c>
+      <c r="K335" s="2" t="n">
+        <v>990.0</v>
+      </c>
+      <c r="L335" s="2" t="s">
+        <v>1629</v>
+      </c>
+      <c r="M335" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N335" s="2" t="s">
         <v>1625</v>
-      </c>
-      <c r="C335" s="2" t="s">
-        <v>1626</v>
-      </c>
-      <c r="D335" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E335" s="2" t="s">
-        <v>1627</v>
-      </c>
-      <c r="F335" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G335" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H335" s="2" t="s">
-        <v>1628</v>
-      </c>
-      <c r="I335" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J335" s="2" t="s">
-        <v>1629</v>
-      </c>
-      <c r="K335" s="2" t="n">
-        <v>982.0</v>
-      </c>
-      <c r="L335" s="2" t="s">
-        <v>1630</v>
-      </c>
-      <c r="M335" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N335" s="2" t="s">
-        <v>1631</v>
       </c>
     </row>
     <row r="336">
@@ -25020,16 +25020,16 @@
         <v>335.0</v>
       </c>
       <c r="B336" s="2" t="s">
+        <v>1630</v>
+      </c>
+      <c r="C336" s="2" t="s">
+        <v>1631</v>
+      </c>
+      <c r="D336" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E336" s="2" t="s">
         <v>1632</v>
-      </c>
-      <c r="C336" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="D336" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E336" s="2" t="s">
-        <v>201</v>
       </c>
       <c r="F336" s="2" t="n">
         <v>0.0</v>
@@ -25047,16 +25047,16 @@
         <v>1634</v>
       </c>
       <c r="K336" s="2" t="n">
-        <v>979.0</v>
+        <v>982.0</v>
       </c>
       <c r="L336" s="2" t="s">
-        <v>201</v>
+        <v>1635</v>
       </c>
       <c r="M336" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N336" s="2" t="s">
-        <v>1635</v>
+        <v>1636</v>
       </c>
     </row>
     <row r="337">
@@ -25064,25 +25064,25 @@
         <v>336.0</v>
       </c>
       <c r="B337" s="2" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="C337" s="2" t="s">
-        <v>1637</v>
+        <v>201</v>
       </c>
       <c r="D337" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E337" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F337" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G337" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H337" s="2" t="s">
         <v>1638</v>
-      </c>
-      <c r="F337" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G337" s="2" t="n">
-        <v>28.0</v>
-      </c>
-      <c r="H337" s="2" t="s">
-        <v>1637</v>
       </c>
       <c r="I337" s="2" t="n">
         <v>0.0</v>
@@ -25091,16 +25091,16 @@
         <v>1639</v>
       </c>
       <c r="K337" s="2" t="n">
-        <v>934.0</v>
+        <v>979.0</v>
       </c>
       <c r="L337" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="M337" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N337" s="2" t="s">
         <v>1640</v>
-      </c>
-      <c r="M337" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N337" s="2" t="s">
-        <v>1641</v>
       </c>
     </row>
     <row r="338">
@@ -25108,25 +25108,25 @@
         <v>337.0</v>
       </c>
       <c r="B338" s="2" t="s">
+        <v>1641</v>
+      </c>
+      <c r="C338" s="2" t="s">
         <v>1642</v>
       </c>
-      <c r="C338" s="2" t="s">
+      <c r="D338" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E338" s="2" t="s">
         <v>1643</v>
       </c>
-      <c r="D338" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E338" s="2" t="s">
-        <v>201</v>
-      </c>
       <c r="F338" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G338" s="2" t="n">
-        <v>0.0</v>
+        <v>28.0</v>
       </c>
       <c r="H338" s="2" t="s">
-        <v>1644</v>
+        <v>1642</v>
       </c>
       <c r="I338" s="2" t="n">
         <v>0.0</v>
@@ -25135,7 +25135,7 @@
         <v>1644</v>
       </c>
       <c r="K338" s="2" t="n">
-        <v>973.0</v>
+        <v>934.0</v>
       </c>
       <c r="L338" s="2" t="s">
         <v>1645</v>
@@ -25161,31 +25161,31 @@
         <v>0.0</v>
       </c>
       <c r="E339" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="F339" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G339" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H339" s="2" t="s">
         <v>1649</v>
       </c>
-      <c r="F339" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G339" s="2" t="n">
-        <v>10.0</v>
-      </c>
-      <c r="H339" s="2" t="s">
-        <v>1648</v>
-      </c>
       <c r="I339" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J339" s="2" t="s">
+        <v>1649</v>
+      </c>
+      <c r="K339" s="2" t="n">
+        <v>973.0</v>
+      </c>
+      <c r="L339" s="2" t="s">
         <v>1650</v>
       </c>
-      <c r="K339" s="2" t="n">
-        <v>926.0</v>
-      </c>
-      <c r="L339" s="2" t="s">
-        <v>1648</v>
-      </c>
       <c r="M339" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="N339" s="2" t="s">
         <v>1651</v>
@@ -41934,7 +41934,7 @@
         <v>0.0</v>
       </c>
       <c r="H720" s="2" t="s">
-        <v>1578</v>
+        <v>1583</v>
       </c>
       <c r="I720" s="2" t="n">
         <v>0.0</v>

</xml_diff>

<commit_message>
Add generated leaderboard data - 2024-05-14T19:10:22
</commit_message>
<xml_diff>
--- a/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
+++ b/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
@@ -173,6 +173,24 @@
     <t>58.38%</t>
   </si>
   <si>
+    <t>22R01A05Q6</t>
+  </si>
+  <si>
+    <t>22r01a05q6</t>
+  </si>
+  <si>
+    <t>22r01a0tkh</t>
+  </si>
+  <si>
+    <t>22R01A05W6</t>
+  </si>
+  <si>
+    <t>shahid24</t>
+  </si>
+  <si>
+    <t>56.27%</t>
+  </si>
+  <si>
     <t>22R01A66D5</t>
   </si>
   <si>
@@ -185,25 +203,7 @@
     <t>Sakethreddy168</t>
   </si>
   <si>
-    <t>56.33%</t>
-  </si>
-  <si>
-    <t>22R01A05Q6</t>
-  </si>
-  <si>
-    <t>22r01a05q6</t>
-  </si>
-  <si>
-    <t>22r01a0tkh</t>
-  </si>
-  <si>
-    <t>22R01A05W6</t>
-  </si>
-  <si>
-    <t>shahid24</t>
-  </si>
-  <si>
-    <t>56.25%</t>
+    <t>54.19%</t>
   </si>
   <si>
     <t>22R01A0531</t>
@@ -281,7 +281,7 @@
     <t>koushikpatel</t>
   </si>
   <si>
-    <t>49.25%</t>
+    <t>49.31%</t>
   </si>
   <si>
     <t>22R01A05A1</t>
@@ -3998,6 +3998,21 @@
     <t>8.58%</t>
   </si>
   <si>
+    <t>22R01A66A2</t>
+  </si>
+  <si>
+    <t>22r01a66a2</t>
+  </si>
+  <si>
+    <t>22r01az40l</t>
+  </si>
+  <si>
+    <t>a22r01a66a2</t>
+  </si>
+  <si>
+    <t>8.57%</t>
+  </si>
+  <si>
     <t>22R01A05C3</t>
   </si>
   <si>
@@ -4097,21 +4112,6 @@
     <t>22r01a6644</t>
   </si>
   <si>
-    <t>22R01A66A2</t>
-  </si>
-  <si>
-    <t>22r01a66a2</t>
-  </si>
-  <si>
-    <t>22r01az40l</t>
-  </si>
-  <si>
-    <t>a22r01a66a2</t>
-  </si>
-  <si>
-    <t>8.13%</t>
-  </si>
-  <si>
     <t>22R01A6211</t>
   </si>
   <si>
@@ -4856,7 +4856,7 @@
     <t>sonikamogili</t>
   </si>
   <si>
-    <t>6.54%</t>
+    <t>6.58%</t>
   </si>
   <si>
     <t>22R01A6679</t>
@@ -10769,37 +10769,37 @@
         <v>54</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>779.0</v>
+        <v>776.0</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>55</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>103.0</v>
+        <v>104.0</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>19.0</v>
+        <v>106.0</v>
       </c>
       <c r="H10" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>1371.0</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>1399.0</v>
+      </c>
+      <c r="L10" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="I10" s="2" t="n">
-        <v>1575.0</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="K10" s="2" t="n">
-        <v>1379.0</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>56</v>
-      </c>
       <c r="M10" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11">
@@ -10807,40 +10807,40 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>776.0</v>
+        <v>779.0</v>
       </c>
       <c r="E11" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>103.0</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>19.0</v>
+      </c>
+      <c r="H11" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="F11" s="2" t="n">
-        <v>104.0</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>104.0</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="I11" s="2" t="n">
-        <v>1371.0</v>
+        <v>1575.0</v>
       </c>
       <c r="J11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>1049.0</v>
+      </c>
+      <c r="L11" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="K11" s="2" t="n">
-        <v>1399.0</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="M11" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="N11" s="2" t="s">
         <v>63</v>
@@ -11042,7 +11042,7 @@
         <v>0.0</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>21.0</v>
+        <v>27.0</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>87</v>
@@ -22300,13 +22300,13 @@
         <v>0.0</v>
       </c>
       <c r="E272" s="2" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="F272" s="2" t="n">
-        <v>10.0</v>
+        <v>0.0</v>
       </c>
       <c r="G272" s="2" t="n">
-        <v>0.0</v>
+        <v>12.0</v>
       </c>
       <c r="H272" s="2" t="s">
         <v>1329</v>
@@ -22315,19 +22315,19 @@
         <v>0.0</v>
       </c>
       <c r="J272" s="2" t="s">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="K272" s="2" t="n">
-        <v>1130.0</v>
+        <v>922.0</v>
       </c>
       <c r="L272" s="2" t="s">
         <v>1329</v>
       </c>
       <c r="M272" s="2" t="n">
-        <v>0.0</v>
+        <v>50.0</v>
       </c>
       <c r="N272" s="2" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="273">
@@ -22335,19 +22335,19 @@
         <v>272.0</v>
       </c>
       <c r="B273" s="2" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>208</v>
+        <v>1334</v>
       </c>
       <c r="D273" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E273" s="2" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="F273" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="G273" s="2" t="n">
         <v>0.0</v>
@@ -22356,13 +22356,13 @@
         <v>1334</v>
       </c>
       <c r="I273" s="2" t="n">
-        <v>1358.0</v>
+        <v>0.0</v>
       </c>
       <c r="J273" s="2" t="s">
         <v>1335</v>
       </c>
       <c r="K273" s="2" t="n">
-        <v>0.0</v>
+        <v>1130.0</v>
       </c>
       <c r="L273" s="2" t="s">
         <v>1334</v>
@@ -22382,7 +22382,7 @@
         <v>1337</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>1338</v>
+        <v>208</v>
       </c>
       <c r="D274" s="2" t="n">
         <v>0.0</v>
@@ -22397,22 +22397,22 @@
         <v>0.0</v>
       </c>
       <c r="H274" s="2" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="I274" s="2" t="n">
-        <v>0.0</v>
+        <v>1358.0</v>
       </c>
       <c r="J274" s="2" t="s">
+        <v>1340</v>
+      </c>
+      <c r="K274" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L274" s="2" t="s">
         <v>1339</v>
       </c>
-      <c r="K274" s="2" t="n">
-        <v>1023.0</v>
-      </c>
-      <c r="L274" s="2" t="s">
-        <v>1340</v>
-      </c>
       <c r="M274" s="2" t="n">
-        <v>35.0</v>
+        <v>0.0</v>
       </c>
       <c r="N274" s="2" t="s">
         <v>1341</v>
@@ -22432,7 +22432,7 @@
         <v>0.0</v>
       </c>
       <c r="E275" s="2" t="s">
-        <v>208</v>
+        <v>1343</v>
       </c>
       <c r="F275" s="2" t="n">
         <v>0.0</v>
@@ -22441,7 +22441,7 @@
         <v>0.0</v>
       </c>
       <c r="H275" s="2" t="s">
-        <v>208</v>
+        <v>1343</v>
       </c>
       <c r="I275" s="2" t="n">
         <v>0.0</v>
@@ -22450,16 +22450,16 @@
         <v>1344</v>
       </c>
       <c r="K275" s="2" t="n">
-        <v>1171.0</v>
+        <v>1023.0</v>
       </c>
       <c r="L275" s="2" t="s">
-        <v>1342</v>
+        <v>1345</v>
       </c>
       <c r="M275" s="2" t="n">
-        <v>14.0</v>
+        <v>35.0</v>
       </c>
       <c r="N275" s="2" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="276">
@@ -22467,19 +22467,19 @@
         <v>275.0</v>
       </c>
       <c r="B276" s="2" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>1347</v>
+        <v>1348</v>
       </c>
       <c r="D276" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="E276" s="2" t="s">
-        <v>1348</v>
+        <v>208</v>
       </c>
       <c r="F276" s="2" t="n">
-        <v>20.0</v>
+        <v>0.0</v>
       </c>
       <c r="G276" s="2" t="n">
         <v>0.0</v>
@@ -22494,13 +22494,13 @@
         <v>1349</v>
       </c>
       <c r="K276" s="2" t="n">
-        <v>889.0</v>
+        <v>1171.0</v>
       </c>
       <c r="L276" s="2" t="s">
         <v>1347</v>
       </c>
       <c r="M276" s="2" t="n">
-        <v>0.0</v>
+        <v>14.0</v>
       </c>
       <c r="N276" s="2" t="s">
         <v>1350</v>
@@ -22523,31 +22523,31 @@
         <v>1353</v>
       </c>
       <c r="F277" s="2" t="n">
-        <v>0.0</v>
+        <v>20.0</v>
       </c>
       <c r="G277" s="2" t="n">
-        <v>5.0</v>
+        <v>0.0</v>
       </c>
       <c r="H277" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="I277" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J277" s="2" t="s">
         <v>1354</v>
       </c>
-      <c r="I277" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J277" s="2" t="s">
+      <c r="K277" s="2" t="n">
+        <v>889.0</v>
+      </c>
+      <c r="L277" s="2" t="s">
         <v>1352</v>
       </c>
-      <c r="K277" s="2" t="n">
-        <v>935.0</v>
-      </c>
-      <c r="L277" s="2" t="s">
+      <c r="M277" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N277" s="2" t="s">
         <v>1355</v>
-      </c>
-      <c r="M277" s="2" t="n">
-        <v>42.0</v>
-      </c>
-      <c r="N277" s="2" t="s">
-        <v>1356</v>
       </c>
     </row>
     <row r="278">
@@ -22555,43 +22555,43 @@
         <v>277.0</v>
       </c>
       <c r="B278" s="2" t="s">
+        <v>1356</v>
+      </c>
+      <c r="C278" s="2" t="s">
         <v>1357</v>
       </c>
-      <c r="C278" s="2" t="s">
+      <c r="D278" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E278" s="2" t="s">
         <v>1358</v>
       </c>
-      <c r="D278" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E278" s="2" t="s">
+      <c r="F278" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G278" s="2" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="H278" s="2" t="s">
         <v>1359</v>
       </c>
-      <c r="F278" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G278" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H278" s="2" t="s">
-        <v>1360</v>
-      </c>
       <c r="I278" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J278" s="2" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="K278" s="2" t="n">
-        <v>1119.0</v>
+        <v>935.0</v>
       </c>
       <c r="L278" s="2" t="s">
         <v>1360</v>
       </c>
       <c r="M278" s="2" t="n">
-        <v>19.0</v>
+        <v>42.0</v>
       </c>
       <c r="N278" s="2" t="s">
-        <v>1356</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="279">
@@ -22599,43 +22599,43 @@
         <v>278.0</v>
       </c>
       <c r="B279" s="2" t="s">
+        <v>1362</v>
+      </c>
+      <c r="C279" s="2" t="s">
+        <v>1363</v>
+      </c>
+      <c r="D279" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="E279" s="2" t="s">
+        <v>1364</v>
+      </c>
+      <c r="F279" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G279" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H279" s="2" t="s">
+        <v>1365</v>
+      </c>
+      <c r="I279" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J279" s="2" t="s">
+        <v>1363</v>
+      </c>
+      <c r="K279" s="2" t="n">
+        <v>1119.0</v>
+      </c>
+      <c r="L279" s="2" t="s">
+        <v>1365</v>
+      </c>
+      <c r="M279" s="2" t="n">
+        <v>19.0</v>
+      </c>
+      <c r="N279" s="2" t="s">
         <v>1361</v>
-      </c>
-      <c r="C279" s="2" t="s">
-        <v>1362</v>
-      </c>
-      <c r="D279" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="E279" s="2" t="s">
-        <v>1363</v>
-      </c>
-      <c r="F279" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G279" s="2" t="n">
-        <v>12.0</v>
-      </c>
-      <c r="H279" s="2" t="s">
-        <v>1362</v>
-      </c>
-      <c r="I279" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J279" s="2" t="s">
-        <v>1364</v>
-      </c>
-      <c r="K279" s="2" t="n">
-        <v>922.0</v>
-      </c>
-      <c r="L279" s="2" t="s">
-        <v>1362</v>
-      </c>
-      <c r="M279" s="2" t="n">
-        <v>41.0</v>
-      </c>
-      <c r="N279" s="2" t="s">
-        <v>1365</v>
       </c>
     </row>
     <row r="280">
@@ -24858,7 +24858,7 @@
         <v>0.0</v>
       </c>
       <c r="G330" s="2" t="n">
-        <v>12.0</v>
+        <v>16.0</v>
       </c>
       <c r="H330" s="2" t="s">
         <v>1612</v>

</xml_diff>

<commit_message>
Add generated leaderboard data - 2024-06-22T19:08:39
</commit_message>
<xml_diff>
--- a/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
+++ b/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
@@ -224,7 +224,7 @@
     <t>22r01a05l1</t>
   </si>
   <si>
-    <t>50.81%</t>
+    <t>50.83%</t>
   </si>
   <si>
     <t>22R01A05G4</t>
@@ -1484,6 +1484,24 @@
     <t>31.25%</t>
   </si>
   <si>
+    <t>22R01A6646</t>
+  </si>
+  <si>
+    <t>Srudeep47</t>
+  </si>
+  <si>
+    <t>22r01a6646</t>
+  </si>
+  <si>
+    <t>Srudeep_47</t>
+  </si>
+  <si>
+    <t>srudeep47</t>
+  </si>
+  <si>
+    <t>31.05%</t>
+  </si>
+  <si>
     <t>22R01A6248</t>
   </si>
   <si>
@@ -1689,24 +1707,6 @@
   </si>
   <si>
     <t>22r01a6652</t>
-  </si>
-  <si>
-    <t>22R01A6646</t>
-  </si>
-  <si>
-    <t>Srudeep47</t>
-  </si>
-  <si>
-    <t>22r01a6646</t>
-  </si>
-  <si>
-    <t>Srudeep_47</t>
-  </si>
-  <si>
-    <t>srudeep47</t>
-  </si>
-  <si>
-    <t>29.61%</t>
   </si>
   <si>
     <t>22R01A6745</t>
@@ -11130,7 +11130,7 @@
         <v>80.0</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>228.0</v>
+        <v>230.0</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>67</v>
@@ -14993,10 +14993,10 @@
         <v>491</v>
       </c>
       <c r="D100" s="2" t="n">
-        <v>603.0</v>
+        <v>745.0</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F100" s="2" t="n">
         <v>0.0</v>
@@ -15005,25 +15005,25 @@
         <v>0.0</v>
       </c>
       <c r="H100" s="2" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>1350.0</v>
+        <v>0.0</v>
       </c>
       <c r="J100" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="K100" s="2" t="n">
+        <v>1018.0</v>
+      </c>
+      <c r="L100" s="2" t="s">
         <v>492</v>
       </c>
-      <c r="K100" s="2" t="n">
-        <v>1157.0</v>
-      </c>
-      <c r="L100" s="2" t="s">
-        <v>490</v>
-      </c>
       <c r="M100" s="2" t="n">
-        <v>0.0</v>
+        <v>117.0</v>
       </c>
       <c r="N100" s="2" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="101">
@@ -15031,34 +15031,34 @@
         <v>100.0</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="D101" s="2" t="n">
-        <v>581.0</v>
+        <v>603.0</v>
       </c>
       <c r="E101" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="F101" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G101" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H101" s="2" t="s">
         <v>496</v>
       </c>
-      <c r="F101" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G101" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H101" s="2" t="s">
-        <v>497</v>
-      </c>
       <c r="I101" s="2" t="n">
-        <v>1476.0</v>
+        <v>1350.0</v>
       </c>
       <c r="J101" s="2" t="s">
         <v>498</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>1122.0</v>
+        <v>1157.0</v>
       </c>
       <c r="L101" s="2" t="s">
         <v>496</v>
@@ -15067,7 +15067,7 @@
         <v>0.0</v>
       </c>
       <c r="N101" s="2" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
     </row>
     <row r="102">
@@ -15075,43 +15075,43 @@
         <v>101.0</v>
       </c>
       <c r="B102" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="D102" s="2" t="n">
+        <v>581.0</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="F102" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G102" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H102" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="I102" s="2" t="n">
+        <v>1476.0</v>
+      </c>
+      <c r="J102" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="K102" s="2" t="n">
+        <v>1122.0</v>
+      </c>
+      <c r="L102" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="M102" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N102" s="2" t="s">
         <v>499</v>
-      </c>
-      <c r="C102" s="2" t="s">
-        <v>500</v>
-      </c>
-      <c r="D102" s="2" t="n">
-        <v>601.0</v>
-      </c>
-      <c r="E102" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="F102" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G102" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H102" s="2" t="s">
-        <v>500</v>
-      </c>
-      <c r="I102" s="2" t="n">
-        <v>1455.0</v>
-      </c>
-      <c r="J102" s="2" t="s">
-        <v>501</v>
-      </c>
-      <c r="K102" s="2" t="n">
-        <v>1045.0</v>
-      </c>
-      <c r="L102" s="2" t="s">
-        <v>500</v>
-      </c>
-      <c r="M102" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N102" s="2" t="s">
-        <v>502</v>
       </c>
     </row>
     <row r="103">
@@ -15119,16 +15119,16 @@
         <v>102.0</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="D103" s="2" t="n">
-        <v>567.0</v>
+        <v>601.0</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>505</v>
+        <v>179</v>
       </c>
       <c r="F103" s="2" t="n">
         <v>0.0</v>
@@ -15140,22 +15140,22 @@
         <v>506</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>1360.0</v>
+        <v>1455.0</v>
       </c>
       <c r="J103" s="2" t="s">
         <v>507</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>1231.0</v>
+        <v>1045.0</v>
       </c>
       <c r="L103" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="M103" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N103" s="2" t="s">
         <v>508</v>
-      </c>
-      <c r="M103" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N103" s="2" t="s">
-        <v>509</v>
       </c>
     </row>
     <row r="104">
@@ -15163,16 +15163,16 @@
         <v>103.0</v>
       </c>
       <c r="B104" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="C104" s="2" t="s">
         <v>510</v>
       </c>
-      <c r="C104" s="2" t="s">
+      <c r="D104" s="2" t="n">
+        <v>567.0</v>
+      </c>
+      <c r="E104" s="2" t="s">
         <v>511</v>
-      </c>
-      <c r="D104" s="2" t="n">
-        <v>589.0</v>
-      </c>
-      <c r="E104" s="2" t="s">
-        <v>512</v>
       </c>
       <c r="F104" s="2" t="n">
         <v>0.0</v>
@@ -15184,22 +15184,22 @@
         <v>512</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>1361.0</v>
+        <v>1360.0</v>
       </c>
       <c r="J104" s="2" t="s">
         <v>513</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>1143.0</v>
+        <v>1231.0</v>
       </c>
       <c r="L104" s="2" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="M104" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N104" s="2" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row r="105">
@@ -15207,16 +15207,16 @@
         <v>104.0</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D105" s="2" t="n">
-        <v>782.0</v>
+        <v>589.0</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="F105" s="2" t="n">
         <v>0.0</v>
@@ -15228,22 +15228,22 @@
         <v>518</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>0.0</v>
+        <v>1361.0</v>
       </c>
       <c r="J105" s="2" t="s">
         <v>519</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>605.0</v>
+        <v>1143.0</v>
       </c>
       <c r="L105" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="M105" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N105" s="2" t="s">
         <v>520</v>
-      </c>
-      <c r="M105" s="2" t="n">
-        <v>137.0</v>
-      </c>
-      <c r="N105" s="2" t="s">
-        <v>521</v>
       </c>
     </row>
     <row r="106">
@@ -15251,43 +15251,43 @@
         <v>105.0</v>
       </c>
       <c r="B106" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="C106" s="2" t="s">
         <v>522</v>
       </c>
-      <c r="C106" s="2" t="s">
+      <c r="D106" s="2" t="n">
+        <v>782.0</v>
+      </c>
+      <c r="E106" s="2" t="s">
         <v>523</v>
       </c>
-      <c r="D106" s="2" t="n">
-        <v>709.0</v>
-      </c>
-      <c r="E106" s="2" t="s">
+      <c r="F106" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G106" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H106" s="2" t="s">
         <v>524</v>
       </c>
-      <c r="F106" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G106" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H106" s="2" t="s">
+      <c r="I106" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J106" s="2" t="s">
         <v>525</v>
       </c>
-      <c r="I106" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J106" s="2" t="s">
-        <v>523</v>
-      </c>
       <c r="K106" s="2" t="n">
-        <v>821.0</v>
+        <v>605.0</v>
       </c>
       <c r="L106" s="2" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="M106" s="2" t="n">
-        <v>143.0</v>
+        <v>137.0</v>
       </c>
       <c r="N106" s="2" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
     </row>
     <row r="107">
@@ -15295,43 +15295,43 @@
         <v>106.0</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="D107" s="2" t="n">
-        <v>574.0</v>
+        <v>709.0</v>
       </c>
       <c r="E107" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="F107" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G107" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H107" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="I107" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J107" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="F107" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G107" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H107" s="2" t="s">
+      <c r="K107" s="2" t="n">
+        <v>821.0</v>
+      </c>
+      <c r="L107" s="2" t="s">
         <v>530</v>
       </c>
-      <c r="I107" s="2" t="n">
-        <v>1356.0</v>
-      </c>
-      <c r="J107" s="2" t="s">
-        <v>530</v>
-      </c>
-      <c r="K107" s="2" t="n">
-        <v>1008.0</v>
-      </c>
-      <c r="L107" s="2" t="s">
-        <v>528</v>
-      </c>
       <c r="M107" s="2" t="n">
-        <v>18.0</v>
+        <v>143.0</v>
       </c>
       <c r="N107" s="2" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row r="108">
@@ -15339,43 +15339,43 @@
         <v>107.0</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="D108" s="2" t="n">
-        <v>593.0</v>
+        <v>574.0</v>
       </c>
       <c r="E108" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="F108" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G108" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H108" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="I108" s="2" t="n">
+        <v>1356.0</v>
+      </c>
+      <c r="J108" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="K108" s="2" t="n">
+        <v>1008.0</v>
+      </c>
+      <c r="L108" s="2" t="s">
         <v>534</v>
       </c>
-      <c r="F108" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G108" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H108" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="I108" s="2" t="n">
-        <v>1410.0</v>
-      </c>
-      <c r="J108" s="2" t="s">
-        <v>535</v>
-      </c>
-      <c r="K108" s="2" t="n">
-        <v>992.0</v>
-      </c>
-      <c r="L108" s="2" t="s">
-        <v>533</v>
-      </c>
       <c r="M108" s="2" t="n">
-        <v>0.0</v>
+        <v>18.0</v>
       </c>
       <c r="N108" s="2" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
     </row>
     <row r="109">
@@ -15383,16 +15383,16 @@
         <v>108.0</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="D109" s="2" t="n">
-        <v>574.0</v>
+        <v>593.0</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="F109" s="2" t="n">
         <v>0.0</v>
@@ -15401,25 +15401,25 @@
         <v>0.0</v>
       </c>
       <c r="H109" s="2" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>1389.0</v>
+        <v>1410.0</v>
       </c>
       <c r="J109" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="K109" s="2" t="n">
+        <v>992.0</v>
+      </c>
+      <c r="L109" s="2" t="s">
         <v>539</v>
       </c>
-      <c r="K109" s="2" t="n">
-        <v>1074.0</v>
-      </c>
-      <c r="L109" s="2" t="s">
-        <v>538</v>
-      </c>
       <c r="M109" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N109" s="2" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
     </row>
     <row r="110">
@@ -15427,43 +15427,43 @@
         <v>109.0</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="D110" s="2" t="n">
-        <v>576.0</v>
+        <v>574.0</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="F110" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G110" s="2" t="n">
-        <v>8.0</v>
+        <v>0.0</v>
       </c>
       <c r="H110" s="2" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>1432.0</v>
+        <v>1389.0</v>
       </c>
       <c r="J110" s="2" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>1007.0</v>
+        <v>1074.0</v>
       </c>
       <c r="L110" s="2" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="M110" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N110" s="2" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
     </row>
     <row r="111">
@@ -15471,37 +15471,37 @@
         <v>110.0</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="D111" s="2" t="n">
-        <v>605.0</v>
+        <v>576.0</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>179</v>
+        <v>548</v>
       </c>
       <c r="F111" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G111" s="2" t="n">
-        <v>0.0</v>
+        <v>8.0</v>
       </c>
       <c r="H111" s="2" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>1435.0</v>
+        <v>1432.0</v>
       </c>
       <c r="J111" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="K111" s="2" t="n">
+        <v>1007.0</v>
+      </c>
+      <c r="L111" s="2" t="s">
         <v>548</v>
-      </c>
-      <c r="K111" s="2" t="n">
-        <v>896.0</v>
-      </c>
-      <c r="L111" s="2" t="s">
-        <v>549</v>
       </c>
       <c r="M111" s="2" t="n">
         <v>0.0</v>
@@ -15521,10 +15521,10 @@
         <v>552</v>
       </c>
       <c r="D112" s="2" t="n">
-        <v>746.0</v>
+        <v>605.0</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>552</v>
+        <v>179</v>
       </c>
       <c r="F112" s="2" t="n">
         <v>0.0</v>
@@ -15533,25 +15533,25 @@
         <v>0.0</v>
       </c>
       <c r="H112" s="2" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>0.0</v>
+        <v>1435.0</v>
       </c>
       <c r="J112" s="2" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>1017.0</v>
+        <v>896.0</v>
       </c>
       <c r="L112" s="2" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="M112" s="2" t="n">
-        <v>90.0</v>
+        <v>0.0</v>
       </c>
       <c r="N112" s="2" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
     </row>
     <row r="113">
@@ -15559,16 +15559,16 @@
         <v>112.0</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="D113" s="2" t="n">
-        <v>578.0</v>
+        <v>746.0</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="F113" s="2" t="n">
         <v>0.0</v>
@@ -15580,22 +15580,22 @@
         <v>558</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>1411.0</v>
+        <v>0.0</v>
       </c>
       <c r="J113" s="2" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>1014.0</v>
+        <v>1017.0</v>
       </c>
       <c r="L113" s="2" t="s">
         <v>558</v>
       </c>
       <c r="M113" s="2" t="n">
-        <v>0.0</v>
+        <v>90.0</v>
       </c>
       <c r="N113" s="2" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
     </row>
     <row r="114">
@@ -15603,43 +15603,43 @@
         <v>113.0</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="C114" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="D114" s="2" t="n">
+        <v>578.0</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="F114" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G114" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H114" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="I114" s="2" t="n">
+        <v>1411.0</v>
+      </c>
+      <c r="J114" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="K114" s="2" t="n">
+        <v>1014.0</v>
+      </c>
+      <c r="L114" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="M114" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N114" s="2" t="s">
         <v>560</v>
-      </c>
-      <c r="D114" s="2" t="n">
-        <v>745.0</v>
-      </c>
-      <c r="E114" s="2" t="s">
-        <v>561</v>
-      </c>
-      <c r="F114" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G114" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H114" s="2" t="s">
-        <v>562</v>
-      </c>
-      <c r="I114" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J114" s="2" t="s">
-        <v>563</v>
-      </c>
-      <c r="K114" s="2" t="n">
-        <v>1018.0</v>
-      </c>
-      <c r="L114" s="2" t="s">
-        <v>561</v>
-      </c>
-      <c r="M114" s="2" t="n">
-        <v>88.0</v>
-      </c>
-      <c r="N114" s="2" t="s">
-        <v>564</v>
       </c>
     </row>
     <row r="115">

</xml_diff>

<commit_message>
Add generated leaderboard data - 2024-06-30T19:09:45
</commit_message>
<xml_diff>
--- a/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
+++ b/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
@@ -140,7 +140,7 @@
     <t>sellilavanya</t>
   </si>
   <si>
-    <t>59.19%</t>
+    <t>59.21%</t>
   </si>
   <si>
     <t>22R01A05C9</t>
@@ -185,7 +185,7 @@
     <t>@KIREET_5L5</t>
   </si>
   <si>
-    <t>51.38%</t>
+    <t>51.42%</t>
   </si>
   <si>
     <t>22R01A05Q6</t>
@@ -3662,7 +3662,7 @@
     <t>vanisathvika</t>
   </si>
   <si>
-    <t>15.65%</t>
+    <t>15.66%</t>
   </si>
   <si>
     <t>22R01A0456</t>
@@ -10928,7 +10928,7 @@
         <v>186.0</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>156.0</v>
+        <v>158.0</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>40</v>
@@ -11060,7 +11060,7 @@
         <v>60.0</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>312.0</v>
+        <v>317.0</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>54</v>
@@ -21400,7 +21400,7 @@
         <v>0.0</v>
       </c>
       <c r="G245" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="H245" s="2" t="s">
         <v>1214</v>

</xml_diff>

<commit_message>
Add generated leaderboard data - 2024-07-14T19:07:53
</commit_message>
<xml_diff>
--- a/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
+++ b/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
@@ -104,6 +104,18 @@
     <t>63.06%</t>
   </si>
   <si>
+    <t>22R01A0531</t>
+  </si>
+  <si>
+    <t>22r01a0531</t>
+  </si>
+  <si>
+    <t>shiva7ganesh</t>
+  </si>
+  <si>
+    <t>60.86%</t>
+  </si>
+  <si>
     <t>22R01A66D5</t>
   </si>
   <si>
@@ -116,18 +128,6 @@
     <t>60.33%</t>
   </si>
   <si>
-    <t>22R01A0531</t>
-  </si>
-  <si>
-    <t>22r01a0531</t>
-  </si>
-  <si>
-    <t>shiva7ganesh</t>
-  </si>
-  <si>
-    <t>59.81%</t>
-  </si>
-  <si>
     <t>22R01A0554</t>
   </si>
   <si>
@@ -200,6 +200,18 @@
     <t>50.83%</t>
   </si>
   <si>
+    <t>22R01A0527</t>
+  </si>
+  <si>
+    <t>anvesh_527</t>
+  </si>
+  <si>
+    <t>anvesh_3</t>
+  </si>
+  <si>
+    <t>49.01%</t>
+  </si>
+  <si>
     <t>22R01A05C9</t>
   </si>
   <si>
@@ -212,18 +224,6 @@
     <t>48.19%</t>
   </si>
   <si>
-    <t>22R01A0527</t>
-  </si>
-  <si>
-    <t>anvesh_527</t>
-  </si>
-  <si>
-    <t>anvesh_3</t>
-  </si>
-  <si>
-    <t>47.95%</t>
-  </si>
-  <si>
     <t>22R01A05Q2</t>
   </si>
   <si>
@@ -1859,6 +1859,21 @@
     <t>28.54%</t>
   </si>
   <si>
+    <t>22R01A0503</t>
+  </si>
+  <si>
+    <t>22r01a0503</t>
+  </si>
+  <si>
+    <t>vaishu_065</t>
+  </si>
+  <si>
+    <t>@22r01a0503</t>
+  </si>
+  <si>
+    <t>28.24%</t>
+  </si>
+  <si>
     <t>22R01A6255</t>
   </si>
   <si>
@@ -2018,21 +2033,6 @@
     <t>27.23%</t>
   </si>
   <si>
-    <t>22R01A0503</t>
-  </si>
-  <si>
-    <t>22r01a0503</t>
-  </si>
-  <si>
-    <t>vaishu_065</t>
-  </si>
-  <si>
-    <t>@22r01a0503</t>
-  </si>
-  <si>
-    <t>27.18%</t>
-  </si>
-  <si>
     <t>22R01A6737</t>
   </si>
   <si>
@@ -4433,7 +4433,7 @@
     <t>a22r01a66a2</t>
   </si>
   <si>
-    <t>12.12%</t>
+    <t>12.14%</t>
   </si>
   <si>
     <t>22R01A0431</t>
@@ -10831,34 +10831,34 @@
         <v>31</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>957.0</v>
+        <v>831.0</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>173.0</v>
+        <v>210.0</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>28.0</v>
+        <v>0.0</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>31</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>1549.0</v>
+        <v>1365.0</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>1288.0</v>
+        <v>1421.0</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>31</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>0.0</v>
+        <v>6.0</v>
       </c>
       <c r="N5" s="2" t="s">
         <v>33</v>
@@ -10875,34 +10875,34 @@
         <v>35</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>831.0</v>
+        <v>957.0</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>200.0</v>
+        <v>173.0</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.0</v>
+        <v>28.0</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>35</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>1365.0</v>
+        <v>1549.0</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>1421.0</v>
+        <v>1288.0</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>35</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>6.0</v>
+        <v>0.0</v>
       </c>
       <c r="N6" s="2" t="s">
         <v>37</v>
@@ -11095,34 +11095,34 @@
         <v>63</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>968.0</v>
+        <v>858.0</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>63</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.0</v>
+        <v>90.0</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>1446.0</v>
+        <v>1311.0</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>64</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>1493.0</v>
+        <v>1418.0</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>109.0</v>
+        <v>16.0</v>
       </c>
       <c r="N11" s="2" t="s">
         <v>65</v>
@@ -11139,34 +11139,34 @@
         <v>67</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>858.0</v>
+        <v>968.0</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>67</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>80.0</v>
+        <v>0.0</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>1311.0</v>
+        <v>1446.0</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>68</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>1418.0</v>
+        <v>1493.0</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>16.0</v>
+        <v>109.0</v>
       </c>
       <c r="N12" s="2" t="s">
         <v>69</v>
@@ -16111,37 +16111,37 @@
         <v>616</v>
       </c>
       <c r="D125" s="2" t="n">
-        <v>577.0</v>
+        <v>352.0</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="F125" s="2" t="n">
-        <v>0.0</v>
+        <v>30.0</v>
       </c>
       <c r="G125" s="2" t="n">
-        <v>0.0</v>
+        <v>35.0</v>
       </c>
       <c r="H125" s="2" t="s">
         <v>616</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>1351.0</v>
+        <v>1353.0</v>
       </c>
       <c r="J125" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="K125" s="2" t="n">
+        <v>1169.0</v>
+      </c>
+      <c r="L125" s="2" t="s">
         <v>618</v>
       </c>
-      <c r="K125" s="2" t="n">
-        <v>843.0</v>
-      </c>
-      <c r="L125" s="2" t="s">
+      <c r="M125" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N125" s="2" t="s">
         <v>619</v>
-      </c>
-      <c r="M125" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N125" s="2" t="s">
-        <v>620</v>
       </c>
     </row>
     <row r="126">
@@ -16149,43 +16149,43 @@
         <v>125.0</v>
       </c>
       <c r="B126" s="2" t="s">
+        <v>620</v>
+      </c>
+      <c r="C126" s="2" t="s">
         <v>621</v>
       </c>
-      <c r="C126" s="2" t="s">
-        <v>622</v>
-      </c>
       <c r="D126" s="2" t="n">
-        <v>345.0</v>
+        <v>577.0</v>
       </c>
       <c r="E126" s="2" t="s">
         <v>622</v>
       </c>
       <c r="F126" s="2" t="n">
-        <v>10.0</v>
+        <v>0.0</v>
       </c>
       <c r="G126" s="2" t="n">
-        <v>14.0</v>
+        <v>0.0</v>
       </c>
       <c r="H126" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="I126" s="2" t="n">
+        <v>1351.0</v>
+      </c>
+      <c r="J126" s="2" t="s">
         <v>623</v>
       </c>
-      <c r="I126" s="2" t="n">
-        <v>1412.0</v>
-      </c>
-      <c r="J126" s="2" t="s">
+      <c r="K126" s="2" t="n">
+        <v>843.0</v>
+      </c>
+      <c r="L126" s="2" t="s">
         <v>624</v>
       </c>
-      <c r="K126" s="2" t="n">
-        <v>1190.0</v>
-      </c>
-      <c r="L126" s="2" t="s">
-        <v>622</v>
-      </c>
       <c r="M126" s="2" t="n">
-        <v>39.0</v>
+        <v>0.0</v>
       </c>
       <c r="N126" s="2" t="s">
-        <v>620</v>
+        <v>625</v>
       </c>
     </row>
     <row r="127">
@@ -16193,43 +16193,43 @@
         <v>126.0</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="D127" s="2" t="n">
-        <v>575.0</v>
+        <v>345.0</v>
       </c>
       <c r="E127" s="2" t="s">
         <v>627</v>
       </c>
       <c r="F127" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="G127" s="2" t="n">
-        <v>0.0</v>
+        <v>14.0</v>
       </c>
       <c r="H127" s="2" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="I127" s="2" t="n">
         <v>1412.0</v>
       </c>
       <c r="J127" s="2" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="K127" s="2" t="n">
-        <v>791.0</v>
+        <v>1190.0</v>
       </c>
       <c r="L127" s="2" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M127" s="2" t="n">
-        <v>0.0</v>
+        <v>39.0</v>
       </c>
       <c r="N127" s="2" t="s">
-        <v>629</v>
+        <v>625</v>
       </c>
     </row>
     <row r="128">
@@ -16243,37 +16243,37 @@
         <v>631</v>
       </c>
       <c r="D128" s="2" t="n">
-        <v>760.0</v>
+        <v>575.0</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="F128" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G128" s="2" t="n">
-        <v>7.0</v>
+        <v>0.0</v>
       </c>
       <c r="H128" s="2" t="s">
         <v>631</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>1461.0</v>
+        <v>1412.0</v>
       </c>
       <c r="J128" s="2" t="s">
         <v>631</v>
       </c>
       <c r="K128" s="2" t="n">
-        <v>0.0</v>
+        <v>791.0</v>
       </c>
       <c r="L128" s="2" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="M128" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N128" s="2" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="129">
@@ -16281,43 +16281,43 @@
         <v>128.0</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="D129" s="2" t="n">
-        <v>519.0</v>
+        <v>760.0</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="F129" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G129" s="2" t="n">
-        <v>0.0</v>
+        <v>7.0</v>
       </c>
       <c r="H129" s="2" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>1410.0</v>
+        <v>1461.0</v>
       </c>
       <c r="J129" s="2" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="K129" s="2" t="n">
-        <v>937.0</v>
+        <v>0.0</v>
       </c>
       <c r="L129" s="2" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="M129" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="N129" s="2" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
     </row>
     <row r="130">
@@ -16325,13 +16325,13 @@
         <v>129.0</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="D130" s="2" t="n">
-        <v>571.0</v>
+        <v>519.0</v>
       </c>
       <c r="E130" s="2" t="s">
         <v>639</v>
@@ -16343,25 +16343,25 @@
         <v>0.0</v>
       </c>
       <c r="H130" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="I130" s="2" t="n">
+        <v>1410.0</v>
+      </c>
+      <c r="J130" s="2" t="s">
         <v>640</v>
       </c>
-      <c r="I130" s="2" t="n">
-        <v>1374.0</v>
-      </c>
-      <c r="J130" s="2" t="s">
+      <c r="K130" s="2" t="n">
+        <v>937.0</v>
+      </c>
+      <c r="L130" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="M130" s="2" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="N130" s="2" t="s">
         <v>641</v>
-      </c>
-      <c r="K130" s="2" t="n">
-        <v>800.0</v>
-      </c>
-      <c r="L130" s="2" t="s">
-        <v>642</v>
-      </c>
-      <c r="M130" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N130" s="2" t="s">
-        <v>643</v>
       </c>
     </row>
     <row r="131">
@@ -16369,43 +16369,43 @@
         <v>130.0</v>
       </c>
       <c r="B131" s="2" t="s">
+        <v>642</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>643</v>
+      </c>
+      <c r="D131" s="2" t="n">
+        <v>571.0</v>
+      </c>
+      <c r="E131" s="2" t="s">
         <v>644</v>
       </c>
-      <c r="C131" s="2" t="s">
+      <c r="F131" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G131" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H131" s="2" t="s">
         <v>645</v>
       </c>
-      <c r="D131" s="2" t="n">
-        <v>359.0</v>
-      </c>
-      <c r="E131" s="2" t="s">
+      <c r="I131" s="2" t="n">
+        <v>1374.0</v>
+      </c>
+      <c r="J131" s="2" t="s">
         <v>646</v>
       </c>
-      <c r="F131" s="2" t="n">
-        <v>30.0</v>
-      </c>
-      <c r="G131" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H131" s="2" t="s">
-        <v>646</v>
-      </c>
-      <c r="I131" s="2" t="n">
-        <v>1451.0</v>
-      </c>
-      <c r="J131" s="2" t="s">
+      <c r="K131" s="2" t="n">
+        <v>800.0</v>
+      </c>
+      <c r="L131" s="2" t="s">
         <v>647</v>
       </c>
-      <c r="K131" s="2" t="n">
-        <v>1043.0</v>
-      </c>
-      <c r="L131" s="2" t="s">
+      <c r="M131" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N131" s="2" t="s">
         <v>648</v>
-      </c>
-      <c r="M131" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N131" s="2" t="s">
-        <v>649</v>
       </c>
     </row>
     <row r="132">
@@ -16413,19 +16413,19 @@
         <v>131.0</v>
       </c>
       <c r="B132" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="C132" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C132" s="2" t="s">
+      <c r="D132" s="2" t="n">
+        <v>359.0</v>
+      </c>
+      <c r="E132" s="2" t="s">
         <v>651</v>
       </c>
-      <c r="D132" s="2" t="n">
-        <v>606.0</v>
-      </c>
-      <c r="E132" s="2" t="s">
-        <v>190</v>
-      </c>
       <c r="F132" s="2" t="n">
-        <v>0.0</v>
+        <v>30.0</v>
       </c>
       <c r="G132" s="2" t="n">
         <v>0.0</v>
@@ -16434,22 +16434,22 @@
         <v>651</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>1378.0</v>
+        <v>1451.0</v>
       </c>
       <c r="J132" s="2" t="s">
         <v>652</v>
       </c>
       <c r="K132" s="2" t="n">
-        <v>639.0</v>
+        <v>1043.0</v>
       </c>
       <c r="L132" s="2" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="M132" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N132" s="2" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
     </row>
     <row r="133">
@@ -16457,16 +16457,16 @@
         <v>132.0</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="D133" s="2" t="n">
-        <v>823.0</v>
+        <v>606.0</v>
       </c>
       <c r="E133" s="2" t="s">
-        <v>655</v>
+        <v>190</v>
       </c>
       <c r="F133" s="2" t="n">
         <v>0.0</v>
@@ -16475,16 +16475,16 @@
         <v>0.0</v>
       </c>
       <c r="H133" s="2" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>0.0</v>
+        <v>1378.0</v>
       </c>
       <c r="J133" s="2" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="K133" s="2" t="n">
-        <v>1093.0</v>
+        <v>639.0</v>
       </c>
       <c r="L133" s="2" t="s">
         <v>656</v>
@@ -16493,7 +16493,7 @@
         <v>0.0</v>
       </c>
       <c r="N133" s="2" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
     </row>
     <row r="134">
@@ -16501,16 +16501,16 @@
         <v>133.0</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="D134" s="2" t="n">
-        <v>801.0</v>
+        <v>823.0</v>
       </c>
       <c r="E134" s="2" t="s">
-        <v>190</v>
+        <v>660</v>
       </c>
       <c r="F134" s="2" t="n">
         <v>0.0</v>
@@ -16519,25 +16519,25 @@
         <v>0.0</v>
       </c>
       <c r="H134" s="2" t="s">
-        <v>190</v>
+        <v>660</v>
       </c>
       <c r="I134" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J134" s="2" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="K134" s="2" t="n">
-        <v>1163.0</v>
+        <v>1093.0</v>
       </c>
       <c r="L134" s="2" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="M134" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N134" s="2" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="135">
@@ -16545,16 +16545,16 @@
         <v>134.0</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="D135" s="2" t="n">
-        <v>414.0</v>
+        <v>801.0</v>
       </c>
       <c r="E135" s="2" t="s">
-        <v>664</v>
+        <v>190</v>
       </c>
       <c r="F135" s="2" t="n">
         <v>0.0</v>
@@ -16563,25 +16563,25 @@
         <v>0.0</v>
       </c>
       <c r="H135" s="2" t="s">
-        <v>665</v>
+        <v>190</v>
       </c>
       <c r="I135" s="2" t="n">
-        <v>1545.0</v>
+        <v>0.0</v>
       </c>
       <c r="J135" s="2" t="s">
         <v>664</v>
       </c>
       <c r="K135" s="2" t="n">
-        <v>1134.0</v>
+        <v>1163.0</v>
       </c>
       <c r="L135" s="2" t="s">
+        <v>665</v>
+      </c>
+      <c r="M135" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N135" s="2" t="s">
         <v>666</v>
-      </c>
-      <c r="M135" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N135" s="2" t="s">
-        <v>667</v>
       </c>
     </row>
     <row r="136">
@@ -16589,34 +16589,34 @@
         <v>135.0</v>
       </c>
       <c r="B136" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="C136" s="2" t="s">
         <v>668</v>
       </c>
-      <c r="C136" s="2" t="s">
-        <v>669</v>
-      </c>
       <c r="D136" s="2" t="n">
-        <v>352.0</v>
+        <v>414.0</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>669</v>
       </c>
       <c r="F136" s="2" t="n">
-        <v>20.0</v>
+        <v>0.0</v>
       </c>
       <c r="G136" s="2" t="n">
-        <v>35.0</v>
+        <v>0.0</v>
       </c>
       <c r="H136" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="I136" s="2" t="n">
+        <v>1545.0</v>
+      </c>
+      <c r="J136" s="2" t="s">
         <v>669</v>
       </c>
-      <c r="I136" s="2" t="n">
-        <v>1353.0</v>
-      </c>
-      <c r="J136" s="2" t="s">
-        <v>670</v>
-      </c>
       <c r="K136" s="2" t="n">
-        <v>1169.0</v>
+        <v>1134.0</v>
       </c>
       <c r="L136" s="2" t="s">
         <v>671</v>
@@ -23644,7 +23644,7 @@
         <v>0.0</v>
       </c>
       <c r="G296" s="2" t="n">
-        <v>67.0</v>
+        <v>69.0</v>
       </c>
       <c r="H296" s="2" t="s">
         <v>1470</v>

</xml_diff>

<commit_message>
Add generated leaderboard data - 2024-07-21T19:09:58
</commit_message>
<xml_diff>
--- a/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
+++ b/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
@@ -13656,7 +13656,7 @@
         <v>254</v>
       </c>
       <c r="M99" s="2" t="n">
-        <v>10.0</v>
+        <v>0.0</v>
       </c>
       <c r="N99" s="2" t="s">
         <v>16</v>
@@ -29959,7 +29959,7 @@
         <v>1257</v>
       </c>
       <c r="F470" s="2" t="n">
-        <v>186.0</v>
+        <v>196.0</v>
       </c>
       <c r="G470" s="2" t="n">
         <v>158.0</v>
@@ -48856,7 +48856,7 @@
         <v>2448</v>
       </c>
       <c r="M899" s="2" t="n">
-        <v>84.0</v>
+        <v>0.0</v>
       </c>
       <c r="N899" s="2" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
Add generated leaderboard data - 2024-07-23T19:09:05
</commit_message>
<xml_diff>
--- a/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
+++ b/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
@@ -698,6 +698,327 @@
     <t>30.11%</t>
   </si>
   <si>
+    <t>22R01A05Q3</t>
+  </si>
+  <si>
+    <t>22r01a05q3</t>
+  </si>
+  <si>
+    <t>cmr_22r01a05q3</t>
+  </si>
+  <si>
+    <t>29.56%</t>
+  </si>
+  <si>
+    <t>22R01A6678</t>
+  </si>
+  <si>
+    <t>22r01a6678</t>
+  </si>
+  <si>
+    <t>cmr_22r01a6678</t>
+  </si>
+  <si>
+    <t>29.52%</t>
+  </si>
+  <si>
+    <t>23R05A6705</t>
+  </si>
+  <si>
+    <t>nishwanth2003</t>
+  </si>
+  <si>
+    <t>nishwanthb5ewu</t>
+  </si>
+  <si>
+    <t>29.48%</t>
+  </si>
+  <si>
+    <t>22R01A0455</t>
+  </si>
+  <si>
+    <t>22r01a0455</t>
+  </si>
+  <si>
+    <t>cmrit26_22r01a0455</t>
+  </si>
+  <si>
+    <t>29.34%</t>
+  </si>
+  <si>
+    <t>22R01A67E0</t>
+  </si>
+  <si>
+    <t>shuboday_1005</t>
+  </si>
+  <si>
+    <t>22r01axwm5</t>
+  </si>
+  <si>
+    <t>@22r01a67e0</t>
+  </si>
+  <si>
+    <t>29.26%</t>
+  </si>
+  <si>
+    <t>22R01A0466</t>
+  </si>
+  <si>
+    <t>allammanisha25</t>
+  </si>
+  <si>
+    <t>Manisha</t>
+  </si>
+  <si>
+    <t>allammaneesha</t>
+  </si>
+  <si>
+    <t>allammaneesha0</t>
+  </si>
+  <si>
+    <t>Cmrit26_22r01a0</t>
+  </si>
+  <si>
+    <t>29.19%</t>
+  </si>
+  <si>
+    <t>22R01A0505</t>
+  </si>
+  <si>
+    <t>22r01a0505</t>
+  </si>
+  <si>
+    <t>eshu5886</t>
+  </si>
+  <si>
+    <t>29.06%</t>
+  </si>
+  <si>
+    <t>22R01A0597</t>
+  </si>
+  <si>
+    <t>22r01a0597</t>
+  </si>
+  <si>
+    <t>SaiKarthikeya</t>
+  </si>
+  <si>
+    <t>xkarthikeya</t>
+  </si>
+  <si>
+    <t>28.94%</t>
+  </si>
+  <si>
+    <t>22R01A6688</t>
+  </si>
+  <si>
+    <t>Sharanya_janke</t>
+  </si>
+  <si>
+    <t>22r01avti2</t>
+  </si>
+  <si>
+    <t>Sharanyareddy6</t>
+  </si>
+  <si>
+    <t>28.91%</t>
+  </si>
+  <si>
+    <t>23R05A6706</t>
+  </si>
+  <si>
+    <t>Hemanth00</t>
+  </si>
+  <si>
+    <t>bhemanthsrinivas</t>
+  </si>
+  <si>
+    <t>Balla_Hemanth_Srinivas</t>
+  </si>
+  <si>
+    <t>bhs23r05a6706</t>
+  </si>
+  <si>
+    <t>28.71%</t>
+  </si>
+  <si>
+    <t>22R01A7345</t>
+  </si>
+  <si>
+    <t>22r01a7345</t>
+  </si>
+  <si>
+    <t>vinuthnanarla1</t>
+  </si>
+  <si>
+    <t>VinuthnaNarla</t>
+  </si>
+  <si>
+    <t>28.69%</t>
+  </si>
+  <si>
+    <t>22R01A05B0</t>
+  </si>
+  <si>
+    <t>hanokpaul5b0</t>
+  </si>
+  <si>
+    <t>22r01a05b0</t>
+  </si>
+  <si>
+    <t>28.63%</t>
+  </si>
+  <si>
+    <t>22R01A7319</t>
+  </si>
+  <si>
+    <t>22r01a7319</t>
+  </si>
+  <si>
+    <t>sanathgampa</t>
+  </si>
+  <si>
+    <t>sanath7319</t>
+  </si>
+  <si>
+    <t>28.54%</t>
+  </si>
+  <si>
+    <t>22R01A04G5</t>
+  </si>
+  <si>
+    <t>22r01a04g5</t>
+  </si>
+  <si>
+    <t>cmr_22r01a04g5</t>
+  </si>
+  <si>
+    <t>28.31%</t>
+  </si>
+  <si>
+    <t>22R01A05L4</t>
+  </si>
+  <si>
+    <t>ajaychelikhani5</t>
+  </si>
+  <si>
+    <t>ajay_5l4</t>
+  </si>
+  <si>
+    <t>22R01A67D0</t>
+  </si>
+  <si>
+    <t>sujith09</t>
+  </si>
+  <si>
+    <t>sujith90</t>
+  </si>
+  <si>
+    <t>22r01a67d0</t>
+  </si>
+  <si>
+    <t>28.26%</t>
+  </si>
+  <si>
+    <t>22R01A66B1</t>
+  </si>
+  <si>
+    <t>mithrareddy</t>
+  </si>
+  <si>
+    <t>22r01ajk2I</t>
+  </si>
+  <si>
+    <t>Mithrareddy_143</t>
+  </si>
+  <si>
+    <t>28.19%</t>
+  </si>
+  <si>
+    <t>23R05A6609</t>
+  </si>
+  <si>
+    <t>s_23r05a6609</t>
+  </si>
+  <si>
+    <t>23r05a6609</t>
+  </si>
+  <si>
+    <t>s23r05a6609</t>
+  </si>
+  <si>
+    <t>28.09%</t>
+  </si>
+  <si>
+    <t>22R01A05N5</t>
+  </si>
+  <si>
+    <t>navaneethmahar</t>
+  </si>
+  <si>
+    <t>22r01a05n5</t>
+  </si>
+  <si>
+    <t>navaneethmahara</t>
+  </si>
+  <si>
+    <t>navaneethmahara1</t>
+  </si>
+  <si>
+    <t>28.05%</t>
+  </si>
+  <si>
+    <t>22R01A6235</t>
+  </si>
+  <si>
+    <t>sricharan_3</t>
+  </si>
+  <si>
+    <t>sricharankmyzm</t>
+  </si>
+  <si>
+    <t>sricharan3</t>
+  </si>
+  <si>
+    <t>sricharankanduk1</t>
+  </si>
+  <si>
+    <t>28.02%</t>
+  </si>
+  <si>
+    <t>22R01A05B3</t>
+  </si>
+  <si>
+    <t>22r01a05b3</t>
+  </si>
+  <si>
+    <t>Anushna_225B3</t>
+  </si>
+  <si>
+    <t>anushna_225b3</t>
+  </si>
+  <si>
+    <t>28.0%</t>
+  </si>
+  <si>
+    <t>22R01A6710</t>
+  </si>
+  <si>
+    <t>22r01a6710</t>
+  </si>
+  <si>
+    <t>22R01A0453</t>
+  </si>
+  <si>
+    <t>22r01a0453</t>
+  </si>
+  <si>
+    <t>Cmr_22r01a0453</t>
+  </si>
+  <si>
+    <t>27.82%</t>
+  </si>
+  <si>
     <t>22R01A05N4</t>
   </si>
   <si>
@@ -710,328 +1031,7 @@
     <t>keerthi_mangali</t>
   </si>
   <si>
-    <t>29.87%</t>
-  </si>
-  <si>
-    <t>22R01A05Q3</t>
-  </si>
-  <si>
-    <t>22r01a05q3</t>
-  </si>
-  <si>
-    <t>cmr_22r01a05q3</t>
-  </si>
-  <si>
-    <t>29.56%</t>
-  </si>
-  <si>
-    <t>22R01A6678</t>
-  </si>
-  <si>
-    <t>22r01a6678</t>
-  </si>
-  <si>
-    <t>cmr_22r01a6678</t>
-  </si>
-  <si>
-    <t>29.52%</t>
-  </si>
-  <si>
-    <t>23R05A6705</t>
-  </si>
-  <si>
-    <t>nishwanth2003</t>
-  </si>
-  <si>
-    <t>nishwanthb5ewu</t>
-  </si>
-  <si>
-    <t>29.48%</t>
-  </si>
-  <si>
-    <t>22R01A0455</t>
-  </si>
-  <si>
-    <t>22r01a0455</t>
-  </si>
-  <si>
-    <t>cmrit26_22r01a0455</t>
-  </si>
-  <si>
-    <t>29.34%</t>
-  </si>
-  <si>
-    <t>22R01A67E0</t>
-  </si>
-  <si>
-    <t>shuboday_1005</t>
-  </si>
-  <si>
-    <t>22r01axwm5</t>
-  </si>
-  <si>
-    <t>@22r01a67e0</t>
-  </si>
-  <si>
-    <t>29.26%</t>
-  </si>
-  <si>
-    <t>22R01A0466</t>
-  </si>
-  <si>
-    <t>allammanisha25</t>
-  </si>
-  <si>
-    <t>Manisha</t>
-  </si>
-  <si>
-    <t>allammaneesha</t>
-  </si>
-  <si>
-    <t>allammaneesha0</t>
-  </si>
-  <si>
-    <t>Cmrit26_22r01a0</t>
-  </si>
-  <si>
-    <t>29.19%</t>
-  </si>
-  <si>
-    <t>22R01A0505</t>
-  </si>
-  <si>
-    <t>22r01a0505</t>
-  </si>
-  <si>
-    <t>eshu5886</t>
-  </si>
-  <si>
-    <t>29.06%</t>
-  </si>
-  <si>
-    <t>22R01A0597</t>
-  </si>
-  <si>
-    <t>22r01a0597</t>
-  </si>
-  <si>
-    <t>SaiKarthikeya</t>
-  </si>
-  <si>
-    <t>xkarthikeya</t>
-  </si>
-  <si>
-    <t>28.94%</t>
-  </si>
-  <si>
-    <t>22R01A6688</t>
-  </si>
-  <si>
-    <t>Sharanya_janke</t>
-  </si>
-  <si>
-    <t>22r01avti2</t>
-  </si>
-  <si>
-    <t>Sharanyareddy6</t>
-  </si>
-  <si>
-    <t>28.91%</t>
-  </si>
-  <si>
-    <t>23R05A6706</t>
-  </si>
-  <si>
-    <t>Hemanth00</t>
-  </si>
-  <si>
-    <t>bhemanthsrinivas</t>
-  </si>
-  <si>
-    <t>Balla_Hemanth_Srinivas</t>
-  </si>
-  <si>
-    <t>bhs23r05a6706</t>
-  </si>
-  <si>
-    <t>28.71%</t>
-  </si>
-  <si>
-    <t>22R01A7345</t>
-  </si>
-  <si>
-    <t>22r01a7345</t>
-  </si>
-  <si>
-    <t>vinuthnanarla1</t>
-  </si>
-  <si>
-    <t>VinuthnaNarla</t>
-  </si>
-  <si>
-    <t>28.69%</t>
-  </si>
-  <si>
-    <t>22R01A05B0</t>
-  </si>
-  <si>
-    <t>hanokpaul5b0</t>
-  </si>
-  <si>
-    <t>22r01a05b0</t>
-  </si>
-  <si>
-    <t>28.63%</t>
-  </si>
-  <si>
-    <t>22R01A7319</t>
-  </si>
-  <si>
-    <t>22r01a7319</t>
-  </si>
-  <si>
-    <t>sanathgampa</t>
-  </si>
-  <si>
-    <t>sanath7319</t>
-  </si>
-  <si>
-    <t>28.54%</t>
-  </si>
-  <si>
-    <t>22R01A04G5</t>
-  </si>
-  <si>
-    <t>22r01a04g5</t>
-  </si>
-  <si>
-    <t>cmr_22r01a04g5</t>
-  </si>
-  <si>
-    <t>28.31%</t>
-  </si>
-  <si>
-    <t>22R01A05L4</t>
-  </si>
-  <si>
-    <t>ajaychelikhani5</t>
-  </si>
-  <si>
-    <t>ajay_5l4</t>
-  </si>
-  <si>
-    <t>22R01A67D0</t>
-  </si>
-  <si>
-    <t>sujith09</t>
-  </si>
-  <si>
-    <t>sujith90</t>
-  </si>
-  <si>
-    <t>22r01a67d0</t>
-  </si>
-  <si>
-    <t>28.26%</t>
-  </si>
-  <si>
-    <t>22R01A66B1</t>
-  </si>
-  <si>
-    <t>mithrareddy</t>
-  </si>
-  <si>
-    <t>22r01ajk2I</t>
-  </si>
-  <si>
-    <t>Mithrareddy_143</t>
-  </si>
-  <si>
-    <t>28.19%</t>
-  </si>
-  <si>
-    <t>23R05A6609</t>
-  </si>
-  <si>
-    <t>s_23r05a6609</t>
-  </si>
-  <si>
-    <t>23r05a6609</t>
-  </si>
-  <si>
-    <t>s23r05a6609</t>
-  </si>
-  <si>
-    <t>28.09%</t>
-  </si>
-  <si>
-    <t>22R01A05N5</t>
-  </si>
-  <si>
-    <t>navaneethmahar</t>
-  </si>
-  <si>
-    <t>22r01a05n5</t>
-  </si>
-  <si>
-    <t>navaneethmahara</t>
-  </si>
-  <si>
-    <t>navaneethmahara1</t>
-  </si>
-  <si>
-    <t>28.05%</t>
-  </si>
-  <si>
-    <t>22R01A6235</t>
-  </si>
-  <si>
-    <t>sricharan_3</t>
-  </si>
-  <si>
-    <t>sricharankmyzm</t>
-  </si>
-  <si>
-    <t>sricharan3</t>
-  </si>
-  <si>
-    <t>sricharankanduk1</t>
-  </si>
-  <si>
-    <t>28.02%</t>
-  </si>
-  <si>
-    <t>22R01A05B3</t>
-  </si>
-  <si>
-    <t>22r01a05b3</t>
-  </si>
-  <si>
-    <t>Anushna_225B3</t>
-  </si>
-  <si>
-    <t>anushna_225b3</t>
-  </si>
-  <si>
-    <t>28.0%</t>
-  </si>
-  <si>
-    <t>22R01A6710</t>
-  </si>
-  <si>
-    <t>22r01a6710</t>
-  </si>
-  <si>
-    <t>22R01A0453</t>
-  </si>
-  <si>
-    <t>22r01a0453</t>
-  </si>
-  <si>
-    <t>Cmr_22r01a0453</t>
-  </si>
-  <si>
-    <t>27.82%</t>
+    <t>27.68%</t>
   </si>
   <si>
     <t>22R01A66H9</t>
@@ -12243,25 +12243,25 @@
         <v>229</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>546.0</v>
+        <v>794.0</v>
       </c>
       <c r="E45" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>11.0</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="I45" s="2" t="n">
+        <v>1377.0</v>
+      </c>
+      <c r="J45" s="2" t="s">
         <v>230</v>
-      </c>
-      <c r="F45" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G45" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H45" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="I45" s="2" t="n">
-        <v>1487.0</v>
-      </c>
-      <c r="J45" s="2" t="s">
-        <v>229</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0.0</v>
@@ -12270,10 +12270,10 @@
         <v>229</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>143.0</v>
+        <v>24.0</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="46">
@@ -12281,43 +12281,43 @@
         <v>45.0</v>
       </c>
       <c r="B46" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="D46" s="2" t="n">
+        <v>844.0</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>1282.0</v>
+      </c>
+      <c r="J46" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="D46" s="2" t="n">
-        <v>794.0</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="F46" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G46" s="2" t="n">
-        <v>11.0</v>
-      </c>
-      <c r="H46" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I46" s="2" t="n">
-        <v>1377.0</v>
-      </c>
-      <c r="J46" s="2" t="s">
+      <c r="K46" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L46" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M46" s="2" t="n">
+        <v>12.0</v>
+      </c>
+      <c r="N46" s="2" t="s">
         <v>235</v>
-      </c>
-      <c r="K46" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="L46" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="M46" s="2" t="n">
-        <v>24.0</v>
-      </c>
-      <c r="N46" s="2" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="47">
@@ -12325,13 +12325,13 @@
         <v>46.0</v>
       </c>
       <c r="B47" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="C47" s="2" t="s">
-        <v>238</v>
-      </c>
       <c r="D47" s="2" t="n">
-        <v>844.0</v>
+        <v>842.0</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>238</v>
@@ -12343,25 +12343,25 @@
         <v>0.0</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>1282.0</v>
+        <v>1381.0</v>
       </c>
       <c r="J47" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="K47" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L47" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="M47" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N47" s="2" t="s">
         <v>239</v>
-      </c>
-      <c r="K47" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="L47" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="M47" s="2" t="n">
-        <v>12.0</v>
-      </c>
-      <c r="N47" s="2" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="48">
@@ -12369,16 +12369,16 @@
         <v>47.0</v>
       </c>
       <c r="B48" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="C48" s="2" t="s">
-        <v>242</v>
-      </c>
       <c r="D48" s="2" t="n">
-        <v>842.0</v>
+        <v>804.0</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="F48" s="2" t="n">
         <v>0.0</v>
@@ -12387,10 +12387,10 @@
         <v>0.0</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>1381.0</v>
+        <v>1423.0</v>
       </c>
       <c r="J48" s="2" t="s">
         <v>242</v>
@@ -12399,13 +12399,13 @@
         <v>0.0</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0.0</v>
+        <v>11.0</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="49">
@@ -12413,13 +12413,13 @@
         <v>48.0</v>
       </c>
       <c r="B49" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="C49" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="C49" s="2" t="s">
-        <v>246</v>
-      </c>
       <c r="D49" s="2" t="n">
-        <v>804.0</v>
+        <v>843.0</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>246</v>
@@ -12431,22 +12431,22 @@
         <v>0.0</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>1423.0</v>
+        <v>1341.0</v>
       </c>
       <c r="J49" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="K49" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L49" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="K49" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="L49" s="2" t="s">
-        <v>246</v>
-      </c>
       <c r="M49" s="2" t="n">
-        <v>11.0</v>
+        <v>0.0</v>
       </c>
       <c r="N49" s="2" t="s">
         <v>248</v>
@@ -12463,7 +12463,7 @@
         <v>250</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>843.0</v>
+        <v>838.0</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>251</v>
@@ -12475,25 +12475,25 @@
         <v>0.0</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>1341.0</v>
+        <v>1351.0</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="M50" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="51">
@@ -12501,28 +12501,28 @@
         <v>50.0</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>838.0</v>
+        <v>716.0</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>0.0</v>
+        <v>27.0</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="H51" s="2" t="s">
         <v>257</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>1351.0</v>
+        <v>1060.0</v>
       </c>
       <c r="J51" s="2" t="s">
         <v>258</v>
@@ -12531,13 +12531,13 @@
         <v>0.0</v>
       </c>
       <c r="L51" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="M51" s="2" t="n">
+        <v>35.0</v>
+      </c>
+      <c r="N51" s="2" t="s">
         <v>259</v>
-      </c>
-      <c r="M51" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N51" s="2" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="52">
@@ -12545,28 +12545,28 @@
         <v>51.0</v>
       </c>
       <c r="B52" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="C52" s="2" t="s">
-        <v>262</v>
-      </c>
       <c r="D52" s="2" t="n">
-        <v>716.0</v>
+        <v>730.0</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>27.0</v>
+        <v>20.0</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>10.0</v>
+        <v>0.0</v>
       </c>
       <c r="H52" s="2" t="s">
         <v>262</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>1060.0</v>
+        <v>1404.0</v>
       </c>
       <c r="J52" s="2" t="s">
         <v>263</v>
@@ -12575,10 +12575,10 @@
         <v>0.0</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>35.0</v>
+        <v>0.0</v>
       </c>
       <c r="N52" s="2" t="s">
         <v>264</v>
@@ -12595,22 +12595,22 @@
         <v>266</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>730.0</v>
+        <v>838.0</v>
       </c>
       <c r="E53" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="H53" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="F53" s="2" t="n">
-        <v>20.0</v>
-      </c>
-      <c r="G53" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>267</v>
-      </c>
       <c r="I53" s="2" t="n">
-        <v>1404.0</v>
+        <v>1304.0</v>
       </c>
       <c r="J53" s="2" t="s">
         <v>268</v>
@@ -12619,7 +12619,7 @@
         <v>0.0</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="M53" s="2" t="n">
         <v>0.0</v>
@@ -12639,7 +12639,7 @@
         <v>271</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>838.0</v>
+        <v>840.0</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>272</v>
@@ -12648,28 +12648,28 @@
         <v>0.0</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>1304.0</v>
+        <v>1248.0</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="55">
@@ -12677,13 +12677,13 @@
         <v>54.0</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>276</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>840.0</v>
+        <v>808.0</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>277</v>
@@ -12695,22 +12695,22 @@
         <v>0.0</v>
       </c>
       <c r="H55" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="I55" s="2" t="n">
+        <v>1383.0</v>
+      </c>
+      <c r="J55" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="I55" s="2" t="n">
-        <v>1248.0</v>
-      </c>
-      <c r="J55" s="2" t="s">
+      <c r="K55" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L55" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="K55" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="L55" s="2" t="s">
-        <v>277</v>
-      </c>
       <c r="M55" s="2" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="N55" s="2" t="s">
         <v>280</v>
@@ -12724,40 +12724,40 @@
         <v>281</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>808.0</v>
+        <v>632.0</v>
       </c>
       <c r="E56" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>20.0</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>12.0</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>1359.0</v>
+      </c>
+      <c r="J56" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="F56" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G56" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H56" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="I56" s="2" t="n">
-        <v>1383.0</v>
-      </c>
-      <c r="J56" s="2" t="s">
+      <c r="K56" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L56" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="K56" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="L56" s="2" t="s">
+      <c r="M56" s="2" t="n">
+        <v>46.0</v>
+      </c>
+      <c r="N56" s="2" t="s">
         <v>284</v>
-      </c>
-      <c r="M56" s="2" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="N56" s="2" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="57">
@@ -12765,40 +12765,40 @@
         <v>56.0</v>
       </c>
       <c r="B57" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="D57" s="2" t="n">
+        <v>783.0</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H57" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="D57" s="2" t="n">
-        <v>632.0</v>
-      </c>
-      <c r="E57" s="2" t="s">
+      <c r="I57" s="2" t="n">
+        <v>1451.0</v>
+      </c>
+      <c r="J57" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="F57" s="2" t="n">
-        <v>20.0</v>
-      </c>
-      <c r="G57" s="2" t="n">
-        <v>12.0</v>
-      </c>
-      <c r="H57" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="I57" s="2" t="n">
-        <v>1359.0</v>
-      </c>
-      <c r="J57" s="2" t="s">
-        <v>287</v>
-      </c>
       <c r="K57" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>46.0</v>
+        <v>2.0</v>
       </c>
       <c r="N57" s="2" t="s">
         <v>289</v>
@@ -12815,25 +12815,25 @@
         <v>291</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>783.0</v>
+        <v>763.0</v>
       </c>
       <c r="E58" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H58" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="F58" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G58" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H58" s="2" t="s">
+      <c r="I58" s="2" t="n">
+        <v>1463.0</v>
+      </c>
+      <c r="J58" s="2" t="s">
         <v>292</v>
-      </c>
-      <c r="I58" s="2" t="n">
-        <v>1451.0</v>
-      </c>
-      <c r="J58" s="2" t="s">
-        <v>293</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>0.0</v>
@@ -12842,10 +12842,10 @@
         <v>291</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>2.0</v>
+        <v>6.0</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="59">
@@ -12853,43 +12853,43 @@
         <v>58.0</v>
       </c>
       <c r="B59" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="C59" s="2" t="s">
+      <c r="D59" s="2" t="n">
+        <v>769.0</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>1315.0</v>
+      </c>
+      <c r="J59" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="D59" s="2" t="n">
-        <v>763.0</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="F59" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G59" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H59" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="I59" s="2" t="n">
-        <v>1463.0</v>
-      </c>
-      <c r="J59" s="2" t="s">
-        <v>297</v>
-      </c>
       <c r="K59" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="M59" s="2" t="n">
-        <v>6.0</v>
+        <v>0.0</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
     </row>
     <row r="60">
@@ -12897,31 +12897,31 @@
         <v>59.0</v>
       </c>
       <c r="B60" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>772.0</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>1353.0</v>
+      </c>
+      <c r="J60" s="2" t="s">
         <v>299</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="D60" s="2" t="n">
-        <v>769.0</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="F60" s="2" t="n">
-        <v>10.0</v>
-      </c>
-      <c r="G60" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="H60" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="I60" s="2" t="n">
-        <v>1315.0</v>
-      </c>
-      <c r="J60" s="2" t="s">
-        <v>301</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0.0</v>
@@ -12930,10 +12930,10 @@
         <v>300</v>
       </c>
       <c r="M60" s="2" t="n">
-        <v>0.0</v>
+        <v>14.0</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
     </row>
     <row r="61">
@@ -12947,10 +12947,10 @@
         <v>303</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>772.0</v>
+        <v>743.0</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F61" s="2" t="n">
         <v>0.0</v>
@@ -12962,10 +12962,10 @@
         <v>303</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>1353.0</v>
+        <v>1371.0</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0.0</v>
@@ -12974,7 +12974,7 @@
         <v>305</v>
       </c>
       <c r="M61" s="2" t="n">
-        <v>14.0</v>
+        <v>25.0</v>
       </c>
       <c r="N61" s="2" t="s">
         <v>306</v>
@@ -12991,7 +12991,7 @@
         <v>308</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>743.0</v>
+        <v>794.0</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>309</v>
@@ -13003,22 +13003,22 @@
         <v>0.0</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>1371.0</v>
+        <v>1350.0</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="M62" s="2" t="n">
-        <v>25.0</v>
+        <v>0.0</v>
       </c>
       <c r="N62" s="2" t="s">
         <v>311</v>
@@ -13035,7 +13035,7 @@
         <v>313</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>794.0</v>
+        <v>729.0</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>314</v>
@@ -13047,25 +13047,25 @@
         <v>0.0</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>1350.0</v>
+        <v>1404.0</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="M63" s="2" t="n">
-        <v>0.0</v>
+        <v>25.0</v>
       </c>
       <c r="N63" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="64">
@@ -13073,16 +13073,16 @@
         <v>63.0</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>729.0</v>
+        <v>776.0</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F64" s="2" t="n">
         <v>0.0</v>
@@ -13091,25 +13091,25 @@
         <v>0.0</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>1404.0</v>
+        <v>1412.0</v>
       </c>
       <c r="J64" s="2" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="L64" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="M64" s="2" t="n">
-        <v>25.0</v>
+        <v>0.0</v>
       </c>
       <c r="N64" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="65">
@@ -13117,19 +13117,19 @@
         <v>64.0</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>776.0</v>
+        <v>635.0</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>325</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0.0</v>
+        <v>20.0</v>
       </c>
       <c r="G65" s="2" t="n">
         <v>0.0</v>
@@ -13138,19 +13138,19 @@
         <v>326</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>1412.0</v>
+        <v>1328.0</v>
       </c>
       <c r="J65" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="L65" s="2" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="M65" s="2" t="n">
-        <v>0.0</v>
+        <v>38.0</v>
       </c>
       <c r="N65" s="2" t="s">
         <v>328</v>
@@ -13167,25 +13167,25 @@
         <v>330</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>635.0</v>
+        <v>760.0</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>330</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>20.0</v>
+        <v>0.0</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>0.0</v>
+        <v>7.0</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>1328.0</v>
+        <v>1461.0</v>
       </c>
       <c r="J66" s="2" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0.0</v>
@@ -13194,10 +13194,10 @@
         <v>330</v>
       </c>
       <c r="M66" s="2" t="n">
-        <v>38.0</v>
+        <v>0.0</v>
       </c>
       <c r="N66" s="2" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
     </row>
     <row r="67">
@@ -13205,43 +13205,43 @@
         <v>66.0</v>
       </c>
       <c r="B67" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>754.0</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="I67" s="2" t="n">
+        <v>1412.0</v>
+      </c>
+      <c r="J67" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="K67" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="L67" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="M67" s="2" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="N67" s="2" t="s">
         <v>334</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="D67" s="2" t="n">
-        <v>760.0</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="F67" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="G67" s="2" t="n">
-        <v>7.0</v>
-      </c>
-      <c r="H67" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="I67" s="2" t="n">
-        <v>1461.0</v>
-      </c>
-      <c r="J67" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="K67" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="L67" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="M67" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N67" s="2" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="68">
@@ -13249,13 +13249,13 @@
         <v>67.0</v>
       </c>
       <c r="B68" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="C68" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="C68" s="2" t="s">
-        <v>337</v>
-      </c>
       <c r="D68" s="2" t="n">
-        <v>754.0</v>
+        <v>458.0</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>337</v>
@@ -13267,22 +13267,22 @@
         <v>0.0</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>1412.0</v>
+        <v>1487.0</v>
       </c>
       <c r="J68" s="2" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="L68" s="2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="M68" s="2" t="n">
-        <v>7.0</v>
+        <v>143.0</v>
       </c>
       <c r="N68" s="2" t="s">
         <v>339</v>

</xml_diff>

<commit_message>
Add generated leaderboard data - 2024-08-03T19:09:18
</commit_message>
<xml_diff>
--- a/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
+++ b/Leaderboards/CurrentCMRITLeaderboard2026.xlsx
@@ -323,7 +323,7 @@
     <t>@msaiteja665</t>
   </si>
   <si>
-    <t>36.32%</t>
+    <t>36.36%</t>
   </si>
   <si>
     <t>22R01A66D1</t>
@@ -11192,7 +11192,7 @@
         <v>158.0</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>188.0</v>
+        <v>192.0</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>100</v>

</xml_diff>